<commit_message>
Actualizar inventario_operaciones.xlsx - 2026-08-01 08:02
</commit_message>
<xml_diff>
--- a/inventario_operaciones.xlsx
+++ b/inventario_operaciones.xlsx
@@ -535,19 +535,19 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>KM041303</t>
+          <t>KM041105</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DROPS HONEY GOLD</t>
+          <t>CORRECTOR DE OJERAS MACADAMIA</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>584</v>
+        <v>726</v>
       </c>
       <c r="D5" t="n">
-        <v>531.7557251908397</v>
+        <v>347.2900763358779</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -563,19 +563,19 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>KM041204</t>
+          <t>KM041103</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LIP GLOSS VOLUMINIZANTE GOLDEN HOUR</t>
+          <t>CORRECTOR DE OJERAS AVELLANA</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>678</v>
+        <v>616</v>
       </c>
       <c r="D6" t="n">
-        <v>166.2595419847328</v>
+        <v>423.8931297709924</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -591,19 +591,19 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KM041105</t>
+          <t>R010303</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CORRECTOR DE OJERAS MACADAMIA</t>
+          <t>SACHET BOMBA ANTIGRASA LA RECETA</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>726</v>
+        <v>587</v>
       </c>
       <c r="D7" t="n">
-        <v>347.2900763358779</v>
+        <v>180</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -619,19 +619,19 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>KM041103</t>
+          <t>KM041202</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CORRECTOR DE OJERAS AVELLANA</t>
+          <t>LIP GLOSS GOLDEN HOUR</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>616</v>
+        <v>655</v>
       </c>
       <c r="D8" t="n">
-        <v>423.8931297709924</v>
+        <v>171.412213740458</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -647,19 +647,19 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>R010303</t>
+          <t>KM041303</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SACHET BOMBA ANTIGRASA LA RECETA</t>
+          <t>DROPS HONEY GOLD</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>587</v>
+        <v>584</v>
       </c>
       <c r="D9" t="n">
-        <v>180</v>
+        <v>531.7557251908397</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -675,19 +675,19 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>KM041202</t>
+          <t>KM041204</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>LIP GLOSS GOLDEN HOUR</t>
+          <t>LIP GLOSS VOLUMINIZANTE GOLDEN HOUR</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>655</v>
+        <v>678</v>
       </c>
       <c r="D10" t="n">
-        <v>171.412213740458</v>
+        <v>166.2595419847328</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -815,19 +815,19 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>D031009</t>
+          <t>K010402</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ESPUMA AUTOBRONCEADORA TON OSCURO DLUCHI</t>
+          <t>PERFUME PARA EL CABELLO CONFIDENTE KABA</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>143</v>
+        <v>322</v>
       </c>
       <c r="D15" t="n">
-        <v>666.412213740458</v>
+        <v>1163.473282442748</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -843,19 +843,19 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>K010402</t>
+          <t>D030601</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PERFUME PARA EL CABELLO CONFIDENTE KABA</t>
+          <t>FRESHING POP AFTER SUN DLUCHI</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>322</v>
+        <v>144</v>
       </c>
       <c r="D16" t="n">
-        <v>1163.473282442748</v>
+        <v>267.9389312977099</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -871,19 +871,19 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>D030601</t>
+          <t>K010403</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>FRESHING POP AFTER SUN DLUCHI</t>
+          <t>PERFUME PARA EL CABELLO SOÑADORA KABA</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>144</v>
+        <v>280</v>
       </c>
       <c r="D17" t="n">
-        <v>267.9389312977099</v>
+        <v>1100.954198473282</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -899,19 +899,19 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>K010403</t>
+          <t>D031009</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PERFUME PARA EL CABELLO SOÑADORA KABA</t>
+          <t>ESPUMA AUTOBRONCEADORA TON OSCURO DLUCHI</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>280</v>
+        <v>143</v>
       </c>
       <c r="D18" t="n">
-        <v>1100.954198473282</v>
+        <v>666.412213740458</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1207,19 +1207,19 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>D031008</t>
+          <t>K020602</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ESPUMA AUTOBRONCEADORA TON MEDIO DLUCHI</t>
+          <t>CREMA FACIAL TENSORA KABA</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>215</v>
+        <v>134</v>
       </c>
       <c r="D29" t="n">
-        <v>1374.389312977099</v>
+        <v>914.0839694656488</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1235,19 +1235,19 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>K020602</t>
+          <t>D031008</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CREMA FACIAL TENSORA KABA</t>
+          <t>ESPUMA AUTOBRONCEADORA TON MEDIO DLUCHI</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>134</v>
+        <v>215</v>
       </c>
       <c r="D30" t="n">
-        <v>914.0839694656488</v>
+        <v>1374.389312977099</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1347,19 +1347,19 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>K010404</t>
+          <t>K020503</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>PERFUME PARA EL CABELLO ARRIESGADA KABA</t>
+          <t>MASCARILLA FACIAL DE BANANO KABA</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>292</v>
+        <v>180</v>
       </c>
       <c r="D34" t="n">
-        <v>1492.557251908397</v>
+        <v>85.87786259541986</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1375,19 +1375,19 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>K020503</t>
+          <t>K020603</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MASCARILLA FACIAL DE BANANO KABA</t>
+          <t>TONICO DE ROSAS KABA</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>180</v>
+        <v>211</v>
       </c>
       <c r="D35" t="n">
-        <v>85.87786259541986</v>
+        <v>975.2290076335877</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1403,19 +1403,19 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>K020603</t>
+          <t>K010301</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>TONICO DE ROSAS KABA</t>
+          <t>TRATAMIENTO CAPILAR REPOLARIZADOR KABA</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>211</v>
+        <v>425</v>
       </c>
       <c r="D36" t="n">
-        <v>975.2290076335877</v>
+        <v>8401.603053435116</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1431,19 +1431,19 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>K010301</t>
+          <t>K010404</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>TRATAMIENTO CAPILAR REPOLARIZADOR KABA</t>
+          <t>PERFUME PARA EL CABELLO ARRIESGADA KABA</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>425</v>
+        <v>292</v>
       </c>
       <c r="D37" t="n">
-        <v>8401.603053435116</v>
+        <v>1492.557251908397</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1655,19 +1655,19 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>KM041104</t>
+          <t>K020506</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CORRECTOR DE OJERAS CARAMELO</t>
+          <t>MASCARILLA FACIAL DE CHOCOLATE KABA</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>618</v>
+        <v>192</v>
       </c>
       <c r="D45" t="n">
-        <v>217.4427480916031</v>
+        <v>138.7786259541985</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1683,19 +1683,19 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>KM041302</t>
+          <t>KM041304</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>DROPS CHAMPAGNE SILVER</t>
+          <t>DROPS PINK GOLD</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>699</v>
+        <v>742</v>
       </c>
       <c r="D46" t="n">
-        <v>192.7099236641222</v>
+        <v>178.6259541984733</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1711,19 +1711,19 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>KM041301</t>
+          <t>KM041104</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>DROPS CHAMPAGNE GOLD</t>
+          <t>CORRECTOR DE OJERAS CARAMELO</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>425</v>
+        <v>618</v>
       </c>
       <c r="D47" t="n">
-        <v>760.8778625954199</v>
+        <v>217.4427480916031</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1739,19 +1739,19 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>K020506</t>
+          <t>KM041302</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>MASCARILLA FACIAL DE CHOCOLATE KABA</t>
+          <t>DROPS CHAMPAGNE SILVER</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>192</v>
+        <v>699</v>
       </c>
       <c r="D48" t="n">
-        <v>138.7786259541985</v>
+        <v>192.7099236641222</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1767,19 +1767,19 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>KM041304</t>
+          <t>KM041301</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>DROPS PINK GOLD</t>
+          <t>DROPS CHAMPAGNE GOLD</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>742</v>
+        <v>425</v>
       </c>
       <c r="D49" t="n">
-        <v>178.6259541984733</v>
+        <v>760.8778625954199</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1823,19 +1823,19 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>KM041106</t>
+          <t>D031004</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CORRECTOR DE OJERAS MIEL</t>
+          <t>MINI BRONCEADOR ZANAHORIA CANELA DLUCHI</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>665</v>
+        <v>607</v>
       </c>
       <c r="D51" t="n">
-        <v>1522.786259541985</v>
+        <v>4990.534351145038</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1851,19 +1851,19 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>KM041308</t>
+          <t>KM041305</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ILUMINADOR PRETTY GIRL</t>
+          <t>ILUMINADOR LIGHTS UP</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>741</v>
+        <v>799</v>
       </c>
       <c r="D52" t="n">
-        <v>148.3969465648855</v>
+        <v>162.824427480916</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1879,19 +1879,19 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>O030501</t>
+          <t>KM041307</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>MANTEQUILLA EXFOLIANTE OMG</t>
+          <t>ILUMINADOR LIQUIDO DAILY SHINE</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>96</v>
+        <v>665</v>
       </c>
       <c r="D53" t="n">
-        <v>4206.641221374046</v>
+        <v>101.6793893129771</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1907,19 +1907,19 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>D031004</t>
+          <t>KM041106</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>MINI BRONCEADOR ZANAHORIA CANELA DLUCHI</t>
+          <t>CORRECTOR DE OJERAS MIEL</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>607</v>
+        <v>665</v>
       </c>
       <c r="D54" t="n">
-        <v>4990.534351145038</v>
+        <v>1522.786259541985</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1935,19 +1935,19 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>KM041305</t>
+          <t>KM041308</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ILUMINADOR LIGHTS UP</t>
+          <t>ILUMINADOR PRETTY GIRL</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>799</v>
+        <v>741</v>
       </c>
       <c r="D55" t="n">
-        <v>162.824427480916</v>
+        <v>148.3969465648855</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1963,19 +1963,19 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>KM041307</t>
+          <t>O030501</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ILUMINADOR LIQUIDO DAILY SHINE</t>
+          <t>MANTEQUILLA EXFOLIANTE OMG</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>665</v>
+        <v>96</v>
       </c>
       <c r="D56" t="n">
-        <v>101.6793893129771</v>
+        <v>4206.641221374046</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -3673,19 +3673,19 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>KM041108</t>
+          <t>KITD0307</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>GEL FIJADOR DE CEJAS</t>
+          <t>KIT DUO BRONCEADORES DLUCHI</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>192</v>
+        <v>24</v>
       </c>
       <c r="D118" t="n">
-        <v>4274.312977099236</v>
+        <v>36.64122137404581</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3701,19 +3701,19 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>KITD0307</t>
+          <t>KM041108</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>KIT DUO BRONCEADORES DLUCHI</t>
+          <t>GEL FIJADOR DE CEJAS</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>24</v>
+        <v>192</v>
       </c>
       <c r="D119" t="n">
-        <v>36.64122137404581</v>
+        <v>4274.312977099236</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3951,19 +3951,19 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>KITK0105</t>
+          <t>KITK0205</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>KIT DE PERFUMES PARA CABELLO KABA</t>
+          <t>KIT PIEL PERFECTA KABA</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>11</v>
+        <v>76</v>
       </c>
       <c r="D128" t="n">
-        <v>20.72519083969465</v>
+        <v>87.25190839694656</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3979,19 +3979,19 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>KITK0205</t>
+          <t>KITK0105</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>KIT PIEL PERFECTA KABA</t>
+          <t>KIT DE PERFUMES PARA CABELLO KABA</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>76</v>
+        <v>11</v>
       </c>
       <c r="D129" t="n">
-        <v>87.25190839694656</v>
+        <v>20.72519083969465</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -4505,19 +4505,19 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>KITO0301</t>
+          <t>KITD0308</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>KIT MANTEQUILLAS OMG</t>
+          <t>MINIKIT DE BRONCEO DLUCHI</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>42</v>
+        <v>113</v>
       </c>
       <c r="D148" t="n">
-        <v>118.5114503816794</v>
+        <v>520.8778625954199</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4533,19 +4533,19 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>KITD0308</t>
+          <t>KITK0109</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>MINIKIT DE BRONCEO DLUCHI</t>
+          <t>KIT RUTINA CAPILAR KABA</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>113</v>
+        <v>30</v>
       </c>
       <c r="D149" t="n">
-        <v>520.8778625954199</v>
+        <v>383.3587786259542</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4561,19 +4561,19 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>KITK0109</t>
+          <t>KITO0301</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>KIT RUTINA CAPILAR KABA</t>
+          <t>KIT MANTEQUILLAS OMG</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="D150" t="n">
-        <v>383.3587786259542</v>
+        <v>118.5114503816794</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4939,16 +4939,16 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>D051501</t>
+          <t>K051501</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>COSMETIQUERA GRANDE DLUCHI</t>
+          <t>COSMETIQUERA GRANDE KABA</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>158</v>
+        <v>85</v>
       </c>
       <c r="D164" t="inlineStr"/>
       <c r="E164" t="inlineStr">
@@ -4965,16 +4965,16 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>K051501</t>
+          <t>D051501</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>COSMETIQUERA GRANDE KABA</t>
+          <t>COSMETIQUERA GRANDE DLUCHI</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>85</v>
+        <v>158</v>
       </c>
       <c r="D165" t="inlineStr"/>
       <c r="E165" t="inlineStr">
@@ -5497,19 +5497,19 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>KM041303</t>
+          <t>KM041105</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>DROPS HONEY GOLD</t>
+          <t>CORRECTOR DE OJERAS MACADAMIA</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>1</v>
+        <v>287</v>
       </c>
       <c r="D185" t="n">
-        <v>531.7557251908397</v>
+        <v>347.2900763358779</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -5525,19 +5525,19 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>KM041204</t>
+          <t>R010303</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>LIP GLOSS VOLUMINIZANTE GOLDEN HOUR</t>
+          <t>SACHET BOMBA ANTIGRASA LA RECETA</t>
         </is>
       </c>
       <c r="C186" t="n">
         <v>1</v>
       </c>
       <c r="D186" t="n">
-        <v>166.2595419847328</v>
+        <v>180</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5553,19 +5553,19 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>KM041105</t>
+          <t>KM041103</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>CORRECTOR DE OJERAS MACADAMIA</t>
+          <t>CORRECTOR DE OJERAS AVELLANA</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>287</v>
+        <v>1</v>
       </c>
       <c r="D187" t="n">
-        <v>347.2900763358779</v>
+        <v>423.8931297709924</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5581,19 +5581,19 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>R010303</t>
+          <t>KM041202</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>SACHET BOMBA ANTIGRASA LA RECETA</t>
+          <t>LIP GLOSS GOLDEN HOUR</t>
         </is>
       </c>
       <c r="C188" t="n">
         <v>1</v>
       </c>
       <c r="D188" t="n">
-        <v>180</v>
+        <v>171.412213740458</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5609,19 +5609,19 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>KM041103</t>
+          <t>KM041303</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>CORRECTOR DE OJERAS AVELLANA</t>
+          <t>DROPS HONEY GOLD</t>
         </is>
       </c>
       <c r="C189" t="n">
         <v>1</v>
       </c>
       <c r="D189" t="n">
-        <v>423.8931297709924</v>
+        <v>531.7557251908397</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5637,19 +5637,19 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>KM041202</t>
+          <t>KM041204</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>LIP GLOSS GOLDEN HOUR</t>
+          <t>LIP GLOSS VOLUMINIZANTE GOLDEN HOUR</t>
         </is>
       </c>
       <c r="C190" t="n">
         <v>1</v>
       </c>
       <c r="D190" t="n">
-        <v>171.412213740458</v>
+        <v>166.2595419847328</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5749,19 +5749,19 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>D031009</t>
+          <t>K010402</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>ESPUMA AUTOBRONCEADORA TON OSCURO DLUCHI</t>
+          <t>PERFUME PARA EL CABELLO CONFIDENTE KABA</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D194" t="n">
-        <v>666.412213740458</v>
+        <v>1163.473282442748</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5777,19 +5777,19 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>K010402</t>
+          <t>D030601</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>PERFUME PARA EL CABELLO CONFIDENTE KABA</t>
+          <t>FRESHING POP AFTER SUN DLUCHI</t>
         </is>
       </c>
       <c r="C195" t="n">
         <v>1</v>
       </c>
       <c r="D195" t="n">
-        <v>1163.473282442748</v>
+        <v>267.9389312977099</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5805,19 +5805,19 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>D030601</t>
+          <t>D031009</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>FRESHING POP AFTER SUN DLUCHI</t>
+          <t>ESPUMA AUTOBRONCEADORA TON OSCURO DLUCHI</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D196" t="n">
-        <v>267.9389312977099</v>
+        <v>666.412213740458</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -6251,19 +6251,19 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>K010404</t>
+          <t>K020503</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>PERFUME PARA EL CABELLO ARRIESGADA KABA</t>
+          <t>MASCARILLA FACIAL DE BANANO KABA</t>
         </is>
       </c>
       <c r="C212" t="n">
         <v>1</v>
       </c>
       <c r="D212" t="n">
-        <v>1492.557251908397</v>
+        <v>85.87786259541986</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -6279,19 +6279,19 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>K020503</t>
+          <t>K020603</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>MASCARILLA FACIAL DE BANANO KABA</t>
+          <t>TONICO DE ROSAS KABA</t>
         </is>
       </c>
       <c r="C213" t="n">
         <v>1</v>
       </c>
       <c r="D213" t="n">
-        <v>85.87786259541986</v>
+        <v>975.2290076335877</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -6307,19 +6307,19 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>K020603</t>
+          <t>K010403</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>TONICO DE ROSAS KABA</t>
+          <t>PERFUME PARA EL CABELLO SOÑADORA KABA</t>
         </is>
       </c>
       <c r="C214" t="n">
         <v>1</v>
       </c>
       <c r="D214" t="n">
-        <v>975.2290076335877</v>
+        <v>1100.954198473282</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -6335,19 +6335,19 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>K010403</t>
+          <t>K010404</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>PERFUME PARA EL CABELLO SOÑADORA KABA</t>
+          <t>PERFUME PARA EL CABELLO ARRIESGADA KABA</t>
         </is>
       </c>
       <c r="C215" t="n">
         <v>1</v>
       </c>
       <c r="D215" t="n">
-        <v>1100.954198473282</v>
+        <v>1492.557251908397</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -6643,19 +6643,19 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>KM041104</t>
+          <t>K020506</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>CORRECTOR DE OJERAS CARAMELO</t>
+          <t>MASCARILLA FACIAL DE CHOCOLATE KABA</t>
         </is>
       </c>
       <c r="C226" t="n">
         <v>1</v>
       </c>
       <c r="D226" t="n">
-        <v>217.4427480916031</v>
+        <v>138.7786259541985</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -6671,19 +6671,19 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>KM041302</t>
+          <t>KM041304</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>DROPS CHAMPAGNE SILVER</t>
+          <t>DROPS PINK GOLD</t>
         </is>
       </c>
       <c r="C227" t="n">
         <v>1</v>
       </c>
       <c r="D227" t="n">
-        <v>192.7099236641222</v>
+        <v>178.6259541984733</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6699,19 +6699,19 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>KM041301</t>
+          <t>KM041104</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>DROPS CHAMPAGNE GOLD</t>
+          <t>CORRECTOR DE OJERAS CARAMELO</t>
         </is>
       </c>
       <c r="C228" t="n">
         <v>1</v>
       </c>
       <c r="D228" t="n">
-        <v>760.8778625954199</v>
+        <v>217.4427480916031</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6727,19 +6727,19 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>K020506</t>
+          <t>KM041302</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>MASCARILLA FACIAL DE CHOCOLATE KABA</t>
+          <t>DROPS CHAMPAGNE SILVER</t>
         </is>
       </c>
       <c r="C229" t="n">
         <v>1</v>
       </c>
       <c r="D229" t="n">
-        <v>138.7786259541985</v>
+        <v>192.7099236641222</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6755,19 +6755,19 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>KM041304</t>
+          <t>KM041301</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>DROPS PINK GOLD</t>
+          <t>DROPS CHAMPAGNE GOLD</t>
         </is>
       </c>
       <c r="C230" t="n">
         <v>1</v>
       </c>
       <c r="D230" t="n">
-        <v>178.6259541984733</v>
+        <v>760.8778625954199</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6783,19 +6783,19 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>KM041106</t>
+          <t>D031004</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>CORRECTOR DE OJERAS MIEL</t>
+          <t>MINI BRONCEADOR ZANAHORIA CANELA DLUCHI</t>
         </is>
       </c>
       <c r="C231" t="n">
-        <v>265</v>
+        <v>1</v>
       </c>
       <c r="D231" t="n">
-        <v>1522.786259541985</v>
+        <v>4990.534351145038</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6811,19 +6811,19 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>KM041308</t>
+          <t>KM041305</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>ILUMINADOR PRETTY GIRL</t>
+          <t>ILUMINADOR LIGHTS UP</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>217</v>
+        <v>1</v>
       </c>
       <c r="D232" t="n">
-        <v>148.3969465648855</v>
+        <v>162.824427480916</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6839,19 +6839,19 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>O030501</t>
+          <t>KM041307</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>MANTEQUILLA EXFOLIANTE OMG</t>
+          <t>ILUMINADOR LIQUIDO DAILY SHINE</t>
         </is>
       </c>
       <c r="C233" t="n">
         <v>1</v>
       </c>
       <c r="D233" t="n">
-        <v>4206.641221374046</v>
+        <v>101.6793893129771</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6867,19 +6867,19 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>D031004</t>
+          <t>KM041106</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>MINI BRONCEADOR ZANAHORIA CANELA DLUCHI</t>
+          <t>CORRECTOR DE OJERAS MIEL</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>1</v>
+        <v>265</v>
       </c>
       <c r="D234" t="n">
-        <v>4990.534351145038</v>
+        <v>1522.786259541985</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6895,19 +6895,19 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>KM041305</t>
+          <t>KM041308</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>ILUMINADOR LIGHTS UP</t>
+          <t>ILUMINADOR PRETTY GIRL</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>1</v>
+        <v>217</v>
       </c>
       <c r="D235" t="n">
-        <v>162.824427480916</v>
+        <v>148.3969465648855</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6923,19 +6923,19 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>KM041307</t>
+          <t>O030501</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>ILUMINADOR LIQUIDO DAILY SHINE</t>
+          <t>MANTEQUILLA EXFOLIANTE OMG</t>
         </is>
       </c>
       <c r="C236" t="n">
         <v>1</v>
       </c>
       <c r="D236" t="n">
-        <v>101.6793893129771</v>
+        <v>4206.641221374046</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -8001,18 +8001,20 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>KM041310</t>
+          <t>K010301</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>RUBOR LIQUIDO DAIQUIRI</t>
+          <t>TRATAMIENTO CAPILAR REPOLARIZADOR KABA</t>
         </is>
       </c>
       <c r="C275" t="n">
         <v>1</v>
       </c>
-      <c r="D275" t="inlineStr"/>
+      <c r="D275" t="n">
+        <v>8401.603053435116</v>
+      </c>
       <c r="E275" t="inlineStr">
         <is>
           <t>PRODUCTO MANUFACTURADO</t>
@@ -8027,20 +8029,18 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>K010301</t>
+          <t>KM041310</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>TRATAMIENTO CAPILAR REPOLARIZADOR KABA</t>
+          <t>RUBOR LIQUIDO DAIQUIRI</t>
         </is>
       </c>
       <c r="C276" t="n">
         <v>1</v>
       </c>
-      <c r="D276" t="n">
-        <v>8401.603053435116</v>
-      </c>
+      <c r="D276" t="inlineStr"/>
       <c r="E276" t="inlineStr">
         <is>
           <t>PRODUCTO MANUFACTURADO</t>
@@ -8693,19 +8693,19 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>KITO0301</t>
+          <t>KITD0308</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>KIT MANTEQUILLAS OMG</t>
+          <t>MINIKIT DE BRONCEO DLUCHI</t>
         </is>
       </c>
       <c r="C300" t="n">
-        <v>48</v>
+        <v>180</v>
       </c>
       <c r="D300" t="n">
-        <v>118.5114503816794</v>
+        <v>520.8778625954199</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -8721,19 +8721,19 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>KITD0308</t>
+          <t>KITK0109</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>MINIKIT DE BRONCEO DLUCHI</t>
+          <t>KIT RUTINA CAPILAR KABA</t>
         </is>
       </c>
       <c r="C301" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="D301" t="n">
-        <v>520.8778625954199</v>
+        <v>383.3587786259542</v>
       </c>
       <c r="E301" t="inlineStr">
         <is>
@@ -8749,19 +8749,19 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>KITK0109</t>
+          <t>KITO0301</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>KIT RUTINA CAPILAR KABA</t>
+          <t>KIT MANTEQUILLAS OMG</t>
         </is>
       </c>
       <c r="C302" t="n">
-        <v>200</v>
+        <v>48</v>
       </c>
       <c r="D302" t="n">
-        <v>383.3587786259542</v>
+        <v>118.5114503816794</v>
       </c>
       <c r="E302" t="inlineStr">
         <is>
@@ -9503,19 +9503,19 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>KM041303</t>
+          <t>R010303</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>DROPS HONEY GOLD</t>
+          <t>SACHET BOMBA ANTIGRASA LA RECETA</t>
         </is>
       </c>
       <c r="C330" t="n">
-        <v>5293</v>
+        <v>3000</v>
       </c>
       <c r="D330" t="n">
-        <v>531.7557251908397</v>
+        <v>180</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -9531,19 +9531,19 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>KM041308</t>
+          <t>KM041202</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>ILUMINADOR PRETTY GIRL</t>
+          <t>LIP GLOSS GOLDEN HOUR</t>
         </is>
       </c>
       <c r="C331" t="n">
-        <v>9802</v>
+        <v>943</v>
       </c>
       <c r="D331" t="n">
-        <v>148.3969465648855</v>
+        <v>171.412213740458</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -9559,19 +9559,19 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>R010303</t>
+          <t>KM041303</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>SACHET BOMBA ANTIGRASA LA RECETA</t>
+          <t>DROPS HONEY GOLD</t>
         </is>
       </c>
       <c r="C332" t="n">
-        <v>3000</v>
+        <v>5293</v>
       </c>
       <c r="D332" t="n">
-        <v>180</v>
+        <v>531.7557251908397</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -9587,19 +9587,19 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>KM041202</t>
+          <t>KM041308</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>LIP GLOSS GOLDEN HOUR</t>
+          <t>ILUMINADOR PRETTY GIRL</t>
         </is>
       </c>
       <c r="C333" t="n">
-        <v>943</v>
+        <v>9802</v>
       </c>
       <c r="D333" t="n">
-        <v>171.412213740458</v>
+        <v>148.3969465648855</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -10225,19 +10225,19 @@
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>K010404</t>
+          <t>K010402</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>PERFUME PARA EL CABELLO ARRIESGADA KABA</t>
+          <t>PERFUME PARA EL CABELLO CONFIDENTE KABA</t>
         </is>
       </c>
       <c r="C357" t="n">
-        <v>2520</v>
+        <v>2016</v>
       </c>
       <c r="D357" t="n">
-        <v>1492.557251908397</v>
+        <v>1163.473282442748</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -10253,19 +10253,19 @@
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>D031009</t>
+          <t>D030601</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>ESPUMA AUTOBRONCEADORA TON OSCURO DLUCHI</t>
+          <t>FRESHING POP AFTER SUN DLUCHI</t>
         </is>
       </c>
       <c r="C358" t="n">
-        <v>1365</v>
+        <v>20434</v>
       </c>
       <c r="D358" t="n">
-        <v>666.412213740458</v>
+        <v>267.9389312977099</v>
       </c>
       <c r="E358" t="inlineStr">
         <is>
@@ -10281,19 +10281,19 @@
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>K010402</t>
+          <t>K010403</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>PERFUME PARA EL CABELLO CONFIDENTE KABA</t>
+          <t>PERFUME PARA EL CABELLO SOÑADORA KABA</t>
         </is>
       </c>
       <c r="C359" t="n">
-        <v>2016</v>
+        <v>5573</v>
       </c>
       <c r="D359" t="n">
-        <v>1163.473282442748</v>
+        <v>1100.954198473282</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -10309,19 +10309,19 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>D030601</t>
+          <t>K010404</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>FRESHING POP AFTER SUN DLUCHI</t>
+          <t>PERFUME PARA EL CABELLO ARRIESGADA KABA</t>
         </is>
       </c>
       <c r="C360" t="n">
-        <v>20434</v>
+        <v>2520</v>
       </c>
       <c r="D360" t="n">
-        <v>267.9389312977099</v>
+        <v>1492.557251908397</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -10337,19 +10337,19 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>K010403</t>
+          <t>D031009</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>PERFUME PARA EL CABELLO SOÑADORA KABA</t>
+          <t>ESPUMA AUTOBRONCEADORA TON OSCURO DLUCHI</t>
         </is>
       </c>
       <c r="C361" t="n">
-        <v>5573</v>
+        <v>1365</v>
       </c>
       <c r="D361" t="n">
-        <v>1100.954198473282</v>
+        <v>666.412213740458</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -11057,19 +11057,19 @@
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>KM041101</t>
+          <t>K010102</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>CORRECTOR DE OJERAS ALMENDRA</t>
+          <t>SHAMPO KIDS KABA</t>
         </is>
       </c>
       <c r="C388" t="n">
-        <v>4248</v>
+        <v>2500</v>
       </c>
       <c r="D388" t="n">
-        <v>2872.786259541985</v>
+        <v>2141.106870229008</v>
       </c>
       <c r="E388" t="inlineStr">
         <is>
@@ -11085,19 +11085,19 @@
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>K010102</t>
+          <t>R010302</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>SHAMPO KIDS KABA</t>
+          <t>TONICO CAPILAR LA RECETA</t>
         </is>
       </c>
       <c r="C389" t="n">
-        <v>2500</v>
+        <v>14006</v>
       </c>
       <c r="D389" t="n">
-        <v>2141.106870229008</v>
+        <v>3218.702290076336</v>
       </c>
       <c r="E389" t="inlineStr">
         <is>
@@ -11113,19 +11113,19 @@
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>R010302</t>
+          <t>K010101</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>TONICO CAPILAR LA RECETA</t>
+          <t>SHAMPO DE CEBOLLA KABA</t>
         </is>
       </c>
       <c r="C390" t="n">
-        <v>14006</v>
+        <v>177726</v>
       </c>
       <c r="D390" t="n">
-        <v>3218.702290076336</v>
+        <v>81409.46564885495</v>
       </c>
       <c r="E390" t="inlineStr">
         <is>
@@ -11141,19 +11141,19 @@
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>K010101</t>
+          <t>KM041101</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>SHAMPO DE CEBOLLA KABA</t>
+          <t>CORRECTOR DE OJERAS ALMENDRA</t>
         </is>
       </c>
       <c r="C391" t="n">
-        <v>177726</v>
+        <v>4248</v>
       </c>
       <c r="D391" t="n">
-        <v>81409.46564885495</v>
+        <v>2872.786259541985</v>
       </c>
       <c r="E391" t="inlineStr">
         <is>
@@ -12353,19 +12353,19 @@
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>KM041302</t>
+          <t>K020506</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>DROPS CHAMPAGNE SILVER</t>
+          <t>MASCARILLA FACIAL DE CHOCOLATE KABA</t>
         </is>
       </c>
       <c r="C437" t="n">
-        <v>6380</v>
+        <v>511</v>
       </c>
       <c r="D437" t="n">
-        <v>192.7099236641222</v>
+        <v>138.7786259541985</v>
       </c>
       <c r="E437" t="inlineStr">
         <is>
@@ -12381,19 +12381,19 @@
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>KM041301</t>
+          <t>KM041304</t>
         </is>
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>DROPS CHAMPAGNE GOLD</t>
+          <t>DROPS PINK GOLD</t>
         </is>
       </c>
       <c r="C438" t="n">
-        <v>4883</v>
+        <v>5472</v>
       </c>
       <c r="D438" t="n">
-        <v>760.8778625954199</v>
+        <v>178.6259541984733</v>
       </c>
       <c r="E438" t="inlineStr">
         <is>
@@ -12409,19 +12409,19 @@
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>K020506</t>
+          <t>KM041302</t>
         </is>
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>MASCARILLA FACIAL DE CHOCOLATE KABA</t>
+          <t>DROPS CHAMPAGNE SILVER</t>
         </is>
       </c>
       <c r="C439" t="n">
-        <v>511</v>
+        <v>6380</v>
       </c>
       <c r="D439" t="n">
-        <v>138.7786259541985</v>
+        <v>192.7099236641222</v>
       </c>
       <c r="E439" t="inlineStr">
         <is>
@@ -12437,19 +12437,19 @@
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>KM041304</t>
+          <t>KM041301</t>
         </is>
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>DROPS PINK GOLD</t>
+          <t>DROPS CHAMPAGNE GOLD</t>
         </is>
       </c>
       <c r="C440" t="n">
-        <v>5472</v>
+        <v>4883</v>
       </c>
       <c r="D440" t="n">
-        <v>178.6259541984733</v>
+        <v>760.8778625954199</v>
       </c>
       <c r="E440" t="inlineStr">
         <is>
@@ -12571,19 +12571,19 @@
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>KM041106</t>
+          <t>D031004</t>
         </is>
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>CORRECTOR DE OJERAS MIEL</t>
+          <t>MINI BRONCEADOR ZANAHORIA CANELA DLUCHI</t>
         </is>
       </c>
       <c r="C445" t="n">
-        <v>2734</v>
+        <v>200</v>
       </c>
       <c r="D445" t="n">
-        <v>1522.786259541985</v>
+        <v>4990.534351145038</v>
       </c>
       <c r="E445" t="inlineStr">
         <is>
@@ -12599,19 +12599,19 @@
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>D031004</t>
+          <t>KM041305</t>
         </is>
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>MINI BRONCEADOR ZANAHORIA CANELA DLUCHI</t>
+          <t>ILUMINADOR LIGHTS UP</t>
         </is>
       </c>
       <c r="C446" t="n">
-        <v>200</v>
+        <v>9468</v>
       </c>
       <c r="D446" t="n">
-        <v>4990.534351145038</v>
+        <v>162.824427480916</v>
       </c>
       <c r="E446" t="inlineStr">
         <is>
@@ -12627,19 +12627,19 @@
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>KM041305</t>
+          <t>KM041307</t>
         </is>
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>ILUMINADOR LIGHTS UP</t>
+          <t>ILUMINADOR LIQUIDO DAILY SHINE</t>
         </is>
       </c>
       <c r="C447" t="n">
-        <v>9468</v>
+        <v>10397</v>
       </c>
       <c r="D447" t="n">
-        <v>162.824427480916</v>
+        <v>101.6793893129771</v>
       </c>
       <c r="E447" t="inlineStr">
         <is>
@@ -12655,19 +12655,19 @@
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>KM041307</t>
+          <t>KM041106</t>
         </is>
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>ILUMINADOR LIQUIDO DAILY SHINE</t>
+          <t>CORRECTOR DE OJERAS MIEL</t>
         </is>
       </c>
       <c r="C448" t="n">
-        <v>10397</v>
+        <v>2734</v>
       </c>
       <c r="D448" t="n">
-        <v>101.6793893129771</v>
+        <v>1522.786259541985</v>
       </c>
       <c r="E448" t="inlineStr">
         <is>
@@ -14995,19 +14995,19 @@
     <row r="535">
       <c r="A535" t="inlineStr">
         <is>
-          <t>KITK0206</t>
+          <t>KITK0301</t>
         </is>
       </c>
       <c r="B535" t="inlineStr">
         <is>
-          <t>KIT RUTINA AM KABA</t>
+          <t>KIT ADIOS MANCHAS KABA</t>
         </is>
       </c>
       <c r="C535" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D535" t="n">
-        <v>34.69465648854962</v>
+        <v>98.58778625954199</v>
       </c>
       <c r="E535" t="inlineStr">
         <is>
@@ -15023,19 +15023,19 @@
     <row r="536">
       <c r="A536" t="inlineStr">
         <is>
-          <t>KITD0304</t>
+          <t>KITK0206</t>
         </is>
       </c>
       <c r="B536" t="inlineStr">
         <is>
-          <t>KIT BRONCEOPERF VAR ZANA CANELA DLUCHI</t>
+          <t>KIT RUTINA AM KABA</t>
         </is>
       </c>
       <c r="C536" t="n">
-        <v>80</v>
+        <v>54</v>
       </c>
       <c r="D536" t="n">
-        <v>116.9083969465649</v>
+        <v>34.69465648854962</v>
       </c>
       <c r="E536" t="inlineStr">
         <is>
@@ -15051,19 +15051,19 @@
     <row r="537">
       <c r="A537" t="inlineStr">
         <is>
-          <t>KITK0301</t>
+          <t>KITD0304</t>
         </is>
       </c>
       <c r="B537" t="inlineStr">
         <is>
-          <t>KIT ADIOS MANCHAS KABA</t>
+          <t>KIT BRONCEOPERF VAR ZANA CANELA DLUCHI</t>
         </is>
       </c>
       <c r="C537" t="n">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="D537" t="n">
-        <v>98.58778625954199</v>
+        <v>116.9083969465649</v>
       </c>
       <c r="E537" t="inlineStr">
         <is>
@@ -15825,21 +15825,21 @@
     <row r="566">
       <c r="A566" t="inlineStr">
         <is>
-          <t>155301</t>
+          <t>ME1011</t>
         </is>
       </c>
       <c r="B566" t="inlineStr">
         <is>
-          <t>ESTOGEL M</t>
+          <t>LOTIÓN PUMP 28/410 SILVER/WHITE</t>
         </is>
       </c>
       <c r="C566" t="n">
-        <v>100000</v>
+        <v>326790</v>
       </c>
       <c r="D566" t="inlineStr"/>
       <c r="E566" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F566" t="inlineStr">
@@ -15851,21 +15851,21 @@
     <row r="567">
       <c r="A567" t="inlineStr">
         <is>
-          <t>ME1011</t>
+          <t>155301</t>
         </is>
       </c>
       <c r="B567" t="inlineStr">
         <is>
-          <t>LOTIÓN PUMP 28/410 SILVER/WHITE</t>
+          <t>ESTOGEL M</t>
         </is>
       </c>
       <c r="C567" t="n">
-        <v>326790</v>
+        <v>100000</v>
       </c>
       <c r="D567" t="inlineStr"/>
       <c r="E567" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F567" t="inlineStr">
@@ -16007,16 +16007,16 @@
     <row r="573">
       <c r="A573" t="inlineStr">
         <is>
-          <t>ME0507</t>
+          <t>ME1028</t>
         </is>
       </c>
       <c r="B573" t="inlineStr">
         <is>
-          <t>BALA TRANSPARENTE 30ML</t>
+          <t>TAPA CON APLICADOR PUNTA PINCEL</t>
         </is>
       </c>
       <c r="C573" t="n">
-        <v>34020</v>
+        <v>14930</v>
       </c>
       <c r="D573" t="inlineStr"/>
       <c r="E573" t="inlineStr">
@@ -16033,16 +16033,16 @@
     <row r="574">
       <c r="A574" t="inlineStr">
         <is>
-          <t>ME1028</t>
+          <t>ME0507</t>
         </is>
       </c>
       <c r="B574" t="inlineStr">
         <is>
-          <t>TAPA CON APLICADOR PUNTA PINCEL</t>
+          <t>BALA TRANSPARENTE 30ML</t>
         </is>
       </c>
       <c r="C574" t="n">
-        <v>14930</v>
+        <v>34020</v>
       </c>
       <c r="D574" t="inlineStr"/>
       <c r="E574" t="inlineStr">
@@ -23149,16 +23149,16 @@
     <row r="883">
       <c r="A883" t="inlineStr">
         <is>
-          <t>D051501</t>
+          <t>K051501</t>
         </is>
       </c>
       <c r="B883" t="inlineStr">
         <is>
-          <t>COSMETIQUERA GRANDE DLUCHI</t>
+          <t>COSMETIQUERA GRANDE KABA</t>
         </is>
       </c>
       <c r="C883" t="n">
-        <v>22000</v>
+        <v>3900</v>
       </c>
       <c r="D883" t="inlineStr"/>
       <c r="E883" t="inlineStr">
@@ -23175,16 +23175,16 @@
     <row r="884">
       <c r="A884" t="inlineStr">
         <is>
-          <t>K051501</t>
+          <t>D051501</t>
         </is>
       </c>
       <c r="B884" t="inlineStr">
         <is>
-          <t>COSMETIQUERA GRANDE KABA</t>
+          <t>COSMETIQUERA GRANDE DLUCHI</t>
         </is>
       </c>
       <c r="C884" t="n">
-        <v>3900</v>
+        <v>22000</v>
       </c>
       <c r="D884" t="inlineStr"/>
       <c r="E884" t="inlineStr">
@@ -36897,21 +36897,21 @@
     <row r="1448">
       <c r="A1448" t="inlineStr">
         <is>
-          <t>314208</t>
+          <t>ME1049</t>
         </is>
       </c>
       <c r="B1448" t="inlineStr">
         <is>
-          <t>GEMTONE AMBER G001</t>
+          <t>TAPA PUSH PULL DORADA ROSCA 24</t>
         </is>
       </c>
       <c r="C1448" t="n">
-        <v>73488</v>
+        <v>3386</v>
       </c>
       <c r="D1448" t="inlineStr"/>
       <c r="E1448" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1448" t="inlineStr">
@@ -36923,21 +36923,21 @@
     <row r="1449">
       <c r="A1449" t="inlineStr">
         <is>
-          <t>ME1049</t>
+          <t>314208</t>
         </is>
       </c>
       <c r="B1449" t="inlineStr">
         <is>
-          <t>TAPA PUSH PULL DORADA ROSCA 24</t>
+          <t>GEMTONE AMBER G001</t>
         </is>
       </c>
       <c r="C1449" t="n">
-        <v>3386</v>
+        <v>73488</v>
       </c>
       <c r="D1449" t="inlineStr"/>
       <c r="E1449" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F1449" t="inlineStr">
@@ -37287,21 +37287,21 @@
     <row r="1463">
       <c r="A1463" t="inlineStr">
         <is>
-          <t>ME0505</t>
+          <t>ET0202</t>
         </is>
       </c>
       <c r="B1463" t="inlineStr">
         <is>
-          <t>BALA TRANSPARENTE 120ML</t>
+          <t>ETIQUETA PERFUME CABELLO ARRIESGAD 120ML</t>
         </is>
       </c>
       <c r="C1463" t="n">
-        <v>2543</v>
+        <v>140</v>
       </c>
       <c r="D1463" t="inlineStr"/>
       <c r="E1463" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1463" t="inlineStr">
@@ -37313,21 +37313,21 @@
     <row r="1464">
       <c r="A1464" t="inlineStr">
         <is>
-          <t>ET0202</t>
+          <t>ME0505</t>
         </is>
       </c>
       <c r="B1464" t="inlineStr">
         <is>
-          <t>ETIQUETA PERFUME CABELLO ARRIESGAD 120ML</t>
+          <t>BALA TRANSPARENTE 120ML</t>
         </is>
       </c>
       <c r="C1464" t="n">
-        <v>140</v>
+        <v>2543</v>
       </c>
       <c r="D1464" t="inlineStr"/>
       <c r="E1464" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1464" t="inlineStr">
@@ -38197,21 +38197,21 @@
     <row r="1498">
       <c r="A1498" t="inlineStr">
         <is>
-          <t>173501</t>
+          <t>ME1043</t>
         </is>
       </c>
       <c r="B1498" t="inlineStr">
         <is>
-          <t>ULTRAMAR U-200 AZUL</t>
+          <t>TAPA FLIP TOP DORADA ROSCA 18</t>
         </is>
       </c>
       <c r="C1498" t="n">
-        <v>5979</v>
+        <v>4500</v>
       </c>
       <c r="D1498" t="inlineStr"/>
       <c r="E1498" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1498" t="inlineStr">
@@ -38223,16 +38223,16 @@
     <row r="1499">
       <c r="A1499" t="inlineStr">
         <is>
-          <t>ME1043</t>
+          <t>ME1044</t>
         </is>
       </c>
       <c r="B1499" t="inlineStr">
         <is>
-          <t>TAPA FLIP TOP DORADA ROSCA 18</t>
+          <t>TAPA FLIP TOP PLATEADA ROSCA 18</t>
         </is>
       </c>
       <c r="C1499" t="n">
-        <v>4500</v>
+        <v>39551</v>
       </c>
       <c r="D1499" t="inlineStr"/>
       <c r="E1499" t="inlineStr">
@@ -38249,21 +38249,21 @@
     <row r="1500">
       <c r="A1500" t="inlineStr">
         <is>
-          <t>ME1044</t>
+          <t>173501</t>
         </is>
       </c>
       <c r="B1500" t="inlineStr">
         <is>
-          <t>TAPA FLIP TOP PLATEADA ROSCA 18</t>
+          <t>ULTRAMAR U-200 AZUL</t>
         </is>
       </c>
       <c r="C1500" t="n">
-        <v>39551</v>
+        <v>5979</v>
       </c>
       <c r="D1500" t="inlineStr"/>
       <c r="E1500" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F1500" t="inlineStr">
@@ -39185,16 +39185,16 @@
     <row r="1536">
       <c r="A1536" t="inlineStr">
         <is>
-          <t>ME0578</t>
+          <t>ME1055</t>
         </is>
       </c>
       <c r="B1536" t="inlineStr">
         <is>
-          <t>ENVASE ROJO RUBOR EN CREMA RUBY</t>
+          <t>TAPA SPRAY VERDE ROSCA 18</t>
         </is>
       </c>
       <c r="C1536" t="n">
-        <v>19980</v>
+        <v>11362</v>
       </c>
       <c r="D1536" t="inlineStr"/>
       <c r="E1536" t="inlineStr">
@@ -39211,16 +39211,16 @@
     <row r="1537">
       <c r="A1537" t="inlineStr">
         <is>
-          <t>ME0579</t>
+          <t>ME0511</t>
         </is>
       </c>
       <c r="B1537" t="inlineStr">
         <is>
-          <t>ENVASE NARANJA RUBOR EN CREMA SALLY</t>
+          <t>ENV PEAD KABA B28 500ML</t>
         </is>
       </c>
       <c r="C1537" t="n">
-        <v>19475</v>
+        <v>28261</v>
       </c>
       <c r="D1537" t="inlineStr"/>
       <c r="E1537" t="inlineStr">
@@ -39237,21 +39237,21 @@
     <row r="1538">
       <c r="A1538" t="inlineStr">
         <is>
-          <t>ME1067</t>
+          <t>ET0253</t>
         </is>
       </c>
       <c r="B1538" t="inlineStr">
         <is>
-          <t>TAPA NARANJA RUBOR EN BARRA SALLY</t>
+          <t>ETIQUETA BRONC DE CHOCOLATE MIEL 45ML</t>
         </is>
       </c>
       <c r="C1538" t="n">
-        <v>19440</v>
+        <v>22864</v>
       </c>
       <c r="D1538" t="inlineStr"/>
       <c r="E1538" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1538" t="inlineStr">
@@ -39263,16 +39263,16 @@
     <row r="1539">
       <c r="A1539" t="inlineStr">
         <is>
-          <t>ME1055</t>
+          <t>ME0578</t>
         </is>
       </c>
       <c r="B1539" t="inlineStr">
         <is>
-          <t>TAPA SPRAY VERDE ROSCA 18</t>
+          <t>ENVASE ROJO RUBOR EN CREMA RUBY</t>
         </is>
       </c>
       <c r="C1539" t="n">
-        <v>11362</v>
+        <v>19980</v>
       </c>
       <c r="D1539" t="inlineStr"/>
       <c r="E1539" t="inlineStr">
@@ -39289,16 +39289,16 @@
     <row r="1540">
       <c r="A1540" t="inlineStr">
         <is>
-          <t>ME0511</t>
+          <t>ME0579</t>
         </is>
       </c>
       <c r="B1540" t="inlineStr">
         <is>
-          <t>ENV PEAD KABA B28 500ML</t>
+          <t>ENVASE NARANJA RUBOR EN CREMA SALLY</t>
         </is>
       </c>
       <c r="C1540" t="n">
-        <v>28261</v>
+        <v>19475</v>
       </c>
       <c r="D1540" t="inlineStr"/>
       <c r="E1540" t="inlineStr">
@@ -39315,21 +39315,21 @@
     <row r="1541">
       <c r="A1541" t="inlineStr">
         <is>
-          <t>ET0253</t>
+          <t>ME1067</t>
         </is>
       </c>
       <c r="B1541" t="inlineStr">
         <is>
-          <t>ETIQUETA BRONC DE CHOCOLATE MIEL 45ML</t>
+          <t>TAPA NARANJA RUBOR EN BARRA SALLY</t>
         </is>
       </c>
       <c r="C1541" t="n">
-        <v>22864</v>
+        <v>19440</v>
       </c>
       <c r="D1541" t="inlineStr"/>
       <c r="E1541" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1541" t="inlineStr">
@@ -39627,16 +39627,16 @@
     <row r="1553">
       <c r="A1553" t="inlineStr">
         <is>
-          <t>ME0504</t>
+          <t>ME1028</t>
         </is>
       </c>
       <c r="B1553" t="inlineStr">
         <is>
-          <t>BALA NEGRA LARGA 120ML</t>
+          <t>TAPA CON APLICADOR PUNTA PINCEL</t>
         </is>
       </c>
       <c r="C1553" t="n">
-        <v>9239</v>
+        <v>15877</v>
       </c>
       <c r="D1553" t="inlineStr"/>
       <c r="E1553" t="inlineStr">
@@ -39653,16 +39653,16 @@
     <row r="1554">
       <c r="A1554" t="inlineStr">
         <is>
-          <t>ME0507</t>
+          <t>ME1059</t>
         </is>
       </c>
       <c r="B1554" t="inlineStr">
         <is>
-          <t>BALA TRANSPARENTE 30ML</t>
+          <t>WIPER ( ESCURRIDOR/BARREDOR) NATURAL</t>
         </is>
       </c>
       <c r="C1554" t="n">
-        <v>24300</v>
+        <v>30387</v>
       </c>
       <c r="D1554" t="inlineStr"/>
       <c r="E1554" t="inlineStr">
@@ -39679,16 +39679,16 @@
     <row r="1555">
       <c r="A1555" t="inlineStr">
         <is>
-          <t>ME1028</t>
+          <t>ME0504</t>
         </is>
       </c>
       <c r="B1555" t="inlineStr">
         <is>
-          <t>TAPA CON APLICADOR PUNTA PINCEL</t>
+          <t>BALA NEGRA LARGA 120ML</t>
         </is>
       </c>
       <c r="C1555" t="n">
-        <v>15877</v>
+        <v>9239</v>
       </c>
       <c r="D1555" t="inlineStr"/>
       <c r="E1555" t="inlineStr">
@@ -39705,16 +39705,16 @@
     <row r="1556">
       <c r="A1556" t="inlineStr">
         <is>
-          <t>ME1059</t>
+          <t>ME0507</t>
         </is>
       </c>
       <c r="B1556" t="inlineStr">
         <is>
-          <t>WIPER ( ESCURRIDOR/BARREDOR) NATURAL</t>
+          <t>BALA TRANSPARENTE 30ML</t>
         </is>
       </c>
       <c r="C1556" t="n">
-        <v>30387</v>
+        <v>24300</v>
       </c>
       <c r="D1556" t="inlineStr"/>
       <c r="E1556" t="inlineStr">
@@ -39913,16 +39913,16 @@
     <row r="1564">
       <c r="A1564" t="inlineStr">
         <is>
-          <t>ME0542</t>
+          <t>ME0523</t>
         </is>
       </c>
       <c r="B1564" t="inlineStr">
         <is>
-          <t>TUBO COLAP ANTOBRONCEADORA 120ML V1</t>
+          <t>ENVASE PVC COLOR BLANCO POCIMA 6ML</t>
         </is>
       </c>
       <c r="C1564" t="n">
-        <v>3493</v>
+        <v>33606</v>
       </c>
       <c r="D1564" t="inlineStr"/>
       <c r="E1564" t="inlineStr">
@@ -39939,16 +39939,16 @@
     <row r="1565">
       <c r="A1565" t="inlineStr">
         <is>
-          <t>ME0545</t>
+          <t>ME0542</t>
         </is>
       </c>
       <c r="B1565" t="inlineStr">
         <is>
-          <t>TUBO COLAP EXFOLIANTE CAPILAR 220GR V1</t>
+          <t>TUBO COLAP ANTOBRONCEADORA 120ML V1</t>
         </is>
       </c>
       <c r="C1565" t="n">
-        <v>1909</v>
+        <v>3493</v>
       </c>
       <c r="D1565" t="inlineStr"/>
       <c r="E1565" t="inlineStr">
@@ -39965,16 +39965,16 @@
     <row r="1566">
       <c r="A1566" t="inlineStr">
         <is>
-          <t>ME0523</t>
+          <t>ME0545</t>
         </is>
       </c>
       <c r="B1566" t="inlineStr">
         <is>
-          <t>ENVASE PVC COLOR BLANCO POCIMA 6ML</t>
+          <t>TUBO COLAP EXFOLIANTE CAPILAR 220GR V1</t>
         </is>
       </c>
       <c r="C1566" t="n">
-        <v>33606</v>
+        <v>1909</v>
       </c>
       <c r="D1566" t="inlineStr"/>
       <c r="E1566" t="inlineStr">
@@ -39991,16 +39991,16 @@
     <row r="1567">
       <c r="A1567" t="inlineStr">
         <is>
-          <t>ME0513</t>
+          <t>ME1040</t>
         </is>
       </c>
       <c r="B1567" t="inlineStr">
         <is>
-          <t>ENVASE APPLE 28/410 TRANSP P30 M1 300ML</t>
+          <t>TAPA FLIP TOP 28 MM ROSADO FLAMENCO</t>
         </is>
       </c>
       <c r="C1567" t="n">
-        <v>9838</v>
+        <v>17344</v>
       </c>
       <c r="D1567" t="inlineStr"/>
       <c r="E1567" t="inlineStr">
@@ -40017,16 +40017,16 @@
     <row r="1568">
       <c r="A1568" t="inlineStr">
         <is>
-          <t>ME1040</t>
+          <t>ME0513</t>
         </is>
       </c>
       <c r="B1568" t="inlineStr">
         <is>
-          <t>TAPA FLIP TOP 28 MM ROSADO FLAMENCO</t>
+          <t>ENVASE APPLE 28/410 TRANSP P30 M1 300ML</t>
         </is>
       </c>
       <c r="C1568" t="n">
-        <v>17344</v>
+        <v>9838</v>
       </c>
       <c r="D1568" t="inlineStr"/>
       <c r="E1568" t="inlineStr">
@@ -41187,16 +41187,16 @@
     <row r="1613">
       <c r="A1613" t="inlineStr">
         <is>
-          <t>ME0544</t>
+          <t>ME0519</t>
         </is>
       </c>
       <c r="B1613" t="inlineStr">
         <is>
-          <t>TUBO COLAP DERMOACLARANTE 60ML V1</t>
+          <t>ENVASE PARA CREMA FACIAL TENSORA</t>
         </is>
       </c>
       <c r="C1613" t="n">
-        <v>8240</v>
+        <v>10009</v>
       </c>
       <c r="D1613" t="inlineStr"/>
       <c r="E1613" t="inlineStr">
@@ -41213,16 +41213,16 @@
     <row r="1614">
       <c r="A1614" t="inlineStr">
         <is>
-          <t>ME0519</t>
+          <t>ME1014</t>
         </is>
       </c>
       <c r="B1614" t="inlineStr">
         <is>
-          <t>ENVASE PARA CREMA FACIAL TENSORA</t>
+          <t>SHINE GREEN COLOR PRESS</t>
         </is>
       </c>
       <c r="C1614" t="n">
-        <v>10009</v>
+        <v>6885</v>
       </c>
       <c r="D1614" t="inlineStr"/>
       <c r="E1614" t="inlineStr">
@@ -41239,16 +41239,16 @@
     <row r="1615">
       <c r="A1615" t="inlineStr">
         <is>
-          <t>ME1014</t>
+          <t>ME0544</t>
         </is>
       </c>
       <c r="B1615" t="inlineStr">
         <is>
-          <t>SHINE GREEN COLOR PRESS</t>
+          <t>TUBO COLAP DERMOACLARANTE 60ML V1</t>
         </is>
       </c>
       <c r="C1615" t="n">
-        <v>6885</v>
+        <v>8240</v>
       </c>
       <c r="D1615" t="inlineStr"/>
       <c r="E1615" t="inlineStr">
@@ -41629,16 +41629,16 @@
     <row r="1630">
       <c r="A1630" t="inlineStr">
         <is>
-          <t>ME1068</t>
+          <t>ME1012</t>
         </is>
       </c>
       <c r="B1630" t="inlineStr">
         <is>
-          <t>TAPA SPRAY BLANCA R 18/410 (DEPILADOR N)</t>
+          <t>BOMBA ENCASQUE DORADA/BRONCEADORES</t>
         </is>
       </c>
       <c r="C1630" t="n">
-        <v>257740</v>
+        <v>27625</v>
       </c>
       <c r="D1630" t="inlineStr"/>
       <c r="E1630" t="inlineStr">
@@ -41655,21 +41655,21 @@
     <row r="1631">
       <c r="A1631" t="inlineStr">
         <is>
-          <t>ME1012</t>
+          <t>ET02138</t>
         </is>
       </c>
       <c r="B1631" t="inlineStr">
         <is>
-          <t>BOMBA ENCASQUE DORADA/BRONCEADORES</t>
+          <t>ETIQUETA KERATINA ALISADOR KABA 500 ML</t>
         </is>
       </c>
       <c r="C1631" t="n">
-        <v>27625</v>
+        <v>2868</v>
       </c>
       <c r="D1631" t="inlineStr"/>
       <c r="E1631" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1631" t="inlineStr">
@@ -41681,16 +41681,16 @@
     <row r="1632">
       <c r="A1632" t="inlineStr">
         <is>
-          <t>ET02138</t>
+          <t>ET02139</t>
         </is>
       </c>
       <c r="B1632" t="inlineStr">
         <is>
-          <t>ETIQUETA KERATINA ALISADOR KABA 500 ML</t>
+          <t>ETIQUETA KERATINA ALISADOR KABA 250 ML</t>
         </is>
       </c>
       <c r="C1632" t="n">
-        <v>2868</v>
+        <v>1368</v>
       </c>
       <c r="D1632" t="inlineStr"/>
       <c r="E1632" t="inlineStr">
@@ -41707,21 +41707,21 @@
     <row r="1633">
       <c r="A1633" t="inlineStr">
         <is>
-          <t>ET02139</t>
+          <t>ME1068</t>
         </is>
       </c>
       <c r="B1633" t="inlineStr">
         <is>
-          <t>ETIQUETA KERATINA ALISADOR KABA 250 ML</t>
+          <t>TAPA SPRAY BLANCA R 18/410 (DEPILADOR N)</t>
         </is>
       </c>
       <c r="C1633" t="n">
-        <v>1368</v>
+        <v>257740</v>
       </c>
       <c r="D1633" t="inlineStr"/>
       <c r="E1633" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1633" t="inlineStr">
@@ -42587,21 +42587,21 @@
     <row r="1667">
       <c r="A1667" t="inlineStr">
         <is>
-          <t>190102</t>
+          <t>ET0202CA</t>
         </is>
       </c>
       <c r="B1667" t="inlineStr">
         <is>
-          <t>CARBÓN ACTIVADO</t>
+          <t>ETIQUETA ILUMINADOR GOLD ROSE CARA</t>
         </is>
       </c>
       <c r="C1667" t="n">
-        <v>500</v>
+        <v>3916</v>
       </c>
       <c r="D1667" t="inlineStr"/>
       <c r="E1667" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1667" t="inlineStr">
@@ -42613,21 +42613,21 @@
     <row r="1668">
       <c r="A1668" t="inlineStr">
         <is>
-          <t>ET0202CA</t>
+          <t>190102</t>
         </is>
       </c>
       <c r="B1668" t="inlineStr">
         <is>
-          <t>ETIQUETA ILUMINADOR GOLD ROSE CARA</t>
+          <t>CARBÓN ACTIVADO</t>
         </is>
       </c>
       <c r="C1668" t="n">
-        <v>3916</v>
+        <v>500</v>
       </c>
       <c r="D1668" t="inlineStr"/>
       <c r="E1668" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F1668" t="inlineStr">
@@ -42691,21 +42691,21 @@
     <row r="1671">
       <c r="A1671" t="inlineStr">
         <is>
-          <t>ME0553</t>
+          <t>ETC0160</t>
         </is>
       </c>
       <c r="B1671" t="inlineStr">
         <is>
-          <t>TUBO COLAP TTO REVITALIZANTE 230ML V1</t>
+          <t>CAJA RUBOR EN CREMA RUBY</t>
         </is>
       </c>
       <c r="C1671" t="n">
-        <v>478</v>
+        <v>10536</v>
       </c>
       <c r="D1671" t="inlineStr"/>
       <c r="E1671" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1671" t="inlineStr">
@@ -42717,16 +42717,16 @@
     <row r="1672">
       <c r="A1672" t="inlineStr">
         <is>
-          <t>ETC0160</t>
+          <t>ETC0161</t>
         </is>
       </c>
       <c r="B1672" t="inlineStr">
         <is>
-          <t>CAJA RUBOR EN CREMA RUBY</t>
+          <t>CAJA RUBOR EN CREMA SALLY</t>
         </is>
       </c>
       <c r="C1672" t="n">
-        <v>10536</v>
+        <v>10328</v>
       </c>
       <c r="D1672" t="inlineStr"/>
       <c r="E1672" t="inlineStr">
@@ -42743,21 +42743,21 @@
     <row r="1673">
       <c r="A1673" t="inlineStr">
         <is>
-          <t>ETC0161</t>
+          <t>ME0553</t>
         </is>
       </c>
       <c r="B1673" t="inlineStr">
         <is>
-          <t>CAJA RUBOR EN CREMA SALLY</t>
+          <t>TUBO COLAP TTO REVITALIZANTE 230ML V1</t>
         </is>
       </c>
       <c r="C1673" t="n">
-        <v>10328</v>
+        <v>478</v>
       </c>
       <c r="D1673" t="inlineStr"/>
       <c r="E1673" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1673" t="inlineStr">
@@ -43289,21 +43289,21 @@
     <row r="1694">
       <c r="A1694" t="inlineStr">
         <is>
-          <t>ME0506</t>
+          <t>ETC0173</t>
         </is>
       </c>
       <c r="B1694" t="inlineStr">
         <is>
-          <t>BALA TRANSPARENTE 260/250 ML</t>
+          <t>CAJA TONICO CAPILAR KABA ROSADA 120ML</t>
         </is>
       </c>
       <c r="C1694" t="n">
-        <v>9784</v>
+        <v>193</v>
       </c>
       <c r="D1694" t="inlineStr"/>
       <c r="E1694" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1694" t="inlineStr">
@@ -43315,21 +43315,21 @@
     <row r="1695">
       <c r="A1695" t="inlineStr">
         <is>
-          <t>ETC0173</t>
+          <t>ME0506</t>
         </is>
       </c>
       <c r="B1695" t="inlineStr">
         <is>
-          <t>CAJA TONICO CAPILAR KABA ROSADA 120ML</t>
+          <t>BALA TRANSPARENTE 260/250 ML</t>
         </is>
       </c>
       <c r="C1695" t="n">
-        <v>193</v>
+        <v>9784</v>
       </c>
       <c r="D1695" t="inlineStr"/>
       <c r="E1695" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1695" t="inlineStr">
@@ -45157,19 +45157,19 @@
     <row r="1764">
       <c r="A1764" t="inlineStr">
         <is>
-          <t>KM041104</t>
+          <t>K020506</t>
         </is>
       </c>
       <c r="B1764" t="inlineStr">
         <is>
-          <t>CORRECTOR DE OJERAS CARAMELO</t>
+          <t>MASCARILLA FACIAL DE CHOCOLATE KABA</t>
         </is>
       </c>
       <c r="C1764" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D1764" t="n">
-        <v>217.4427480916031</v>
+        <v>138.7786259541985</v>
       </c>
       <c r="E1764" t="inlineStr">
         <is>
@@ -45185,19 +45185,19 @@
     <row r="1765">
       <c r="A1765" t="inlineStr">
         <is>
-          <t>K020506</t>
+          <t>KM041304</t>
         </is>
       </c>
       <c r="B1765" t="inlineStr">
         <is>
-          <t>MASCARILLA FACIAL DE CHOCOLATE KABA</t>
+          <t>DROPS PINK GOLD</t>
         </is>
       </c>
       <c r="C1765" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D1765" t="n">
-        <v>138.7786259541985</v>
+        <v>178.6259541984733</v>
       </c>
       <c r="E1765" t="inlineStr">
         <is>
@@ -45213,19 +45213,19 @@
     <row r="1766">
       <c r="A1766" t="inlineStr">
         <is>
-          <t>KM041304</t>
+          <t>KM041104</t>
         </is>
       </c>
       <c r="B1766" t="inlineStr">
         <is>
-          <t>DROPS PINK GOLD</t>
+          <t>CORRECTOR DE OJERAS CARAMELO</t>
         </is>
       </c>
       <c r="C1766" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D1766" t="n">
-        <v>178.6259541984733</v>
+        <v>217.4427480916031</v>
       </c>
       <c r="E1766" t="inlineStr">
         <is>
@@ -45269,19 +45269,19 @@
     <row r="1768">
       <c r="A1768" t="inlineStr">
         <is>
-          <t>O030501</t>
+          <t>O030801</t>
         </is>
       </c>
       <c r="B1768" t="inlineStr">
         <is>
-          <t>MANTEQUILLA EXFOLIANTE OMG</t>
+          <t>DEPILADOR INSTANTANEO OMG</t>
         </is>
       </c>
       <c r="C1768" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D1768" t="n">
-        <v>4206.641221374046</v>
+        <v>38473.96946564886</v>
       </c>
       <c r="E1768" t="inlineStr">
         <is>
@@ -45297,19 +45297,19 @@
     <row r="1769">
       <c r="A1769" t="inlineStr">
         <is>
-          <t>O030801</t>
+          <t>O030501</t>
         </is>
       </c>
       <c r="B1769" t="inlineStr">
         <is>
-          <t>DEPILADOR INSTANTANEO OMG</t>
+          <t>MANTEQUILLA EXFOLIANTE OMG</t>
         </is>
       </c>
       <c r="C1769" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D1769" t="n">
-        <v>38473.96946564886</v>
+        <v>4206.641221374046</v>
       </c>
       <c r="E1769" t="inlineStr">
         <is>
@@ -45549,19 +45549,19 @@
     <row r="1778">
       <c r="A1778" t="inlineStr">
         <is>
-          <t>KM041108</t>
+          <t>K020507</t>
         </is>
       </c>
       <c r="B1778" t="inlineStr">
         <is>
-          <t>GEL FIJADOR DE CEJAS</t>
+          <t>MASCARILLA FACIAL DE FRUTOS ROJOS KABA</t>
         </is>
       </c>
       <c r="C1778" t="n">
         <v>1</v>
       </c>
       <c r="D1778" t="n">
-        <v>4274.312977099236</v>
+        <v>239.0839694656489</v>
       </c>
       <c r="E1778" t="inlineStr">
         <is>
@@ -45577,19 +45577,19 @@
     <row r="1779">
       <c r="A1779" t="inlineStr">
         <is>
-          <t>K020507</t>
+          <t>KM041108</t>
         </is>
       </c>
       <c r="B1779" t="inlineStr">
         <is>
-          <t>MASCARILLA FACIAL DE FRUTOS ROJOS KABA</t>
+          <t>GEL FIJADOR DE CEJAS</t>
         </is>
       </c>
       <c r="C1779" t="n">
         <v>1</v>
       </c>
       <c r="D1779" t="n">
-        <v>239.0839694656489</v>
+        <v>4274.312977099236</v>
       </c>
       <c r="E1779" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Actualizar inventario_operaciones.xlsx (solo-inventario) - 2026-08-01 12:00
</commit_message>
<xml_diff>
--- a/inventario_operaciones.xlsx
+++ b/inventario_operaciones.xlsx
@@ -15825,21 +15825,21 @@
     <row r="566">
       <c r="A566" t="inlineStr">
         <is>
-          <t>ME1011</t>
+          <t>155301</t>
         </is>
       </c>
       <c r="B566" t="inlineStr">
         <is>
-          <t>LOTIÓN PUMP 28/410 SILVER/WHITE</t>
+          <t>ESTOGEL M</t>
         </is>
       </c>
       <c r="C566" t="n">
-        <v>326790</v>
+        <v>100000</v>
       </c>
       <c r="D566" t="inlineStr"/>
       <c r="E566" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F566" t="inlineStr">
@@ -15851,21 +15851,21 @@
     <row r="567">
       <c r="A567" t="inlineStr">
         <is>
-          <t>155301</t>
+          <t>ME1011</t>
         </is>
       </c>
       <c r="B567" t="inlineStr">
         <is>
-          <t>ESTOGEL M</t>
+          <t>LOTIÓN PUMP 28/410 SILVER/WHITE</t>
         </is>
       </c>
       <c r="C567" t="n">
-        <v>100000</v>
+        <v>326790</v>
       </c>
       <c r="D567" t="inlineStr"/>
       <c r="E567" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F567" t="inlineStr">
@@ -16007,16 +16007,16 @@
     <row r="573">
       <c r="A573" t="inlineStr">
         <is>
-          <t>ME1028</t>
+          <t>ME0507</t>
         </is>
       </c>
       <c r="B573" t="inlineStr">
         <is>
-          <t>TAPA CON APLICADOR PUNTA PINCEL</t>
+          <t>BALA TRANSPARENTE 30ML</t>
         </is>
       </c>
       <c r="C573" t="n">
-        <v>14930</v>
+        <v>34020</v>
       </c>
       <c r="D573" t="inlineStr"/>
       <c r="E573" t="inlineStr">
@@ -16033,16 +16033,16 @@
     <row r="574">
       <c r="A574" t="inlineStr">
         <is>
-          <t>ME0507</t>
+          <t>ME1028</t>
         </is>
       </c>
       <c r="B574" t="inlineStr">
         <is>
-          <t>BALA TRANSPARENTE 30ML</t>
+          <t>TAPA CON APLICADOR PUNTA PINCEL</t>
         </is>
       </c>
       <c r="C574" t="n">
-        <v>34020</v>
+        <v>14930</v>
       </c>
       <c r="D574" t="inlineStr"/>
       <c r="E574" t="inlineStr">
@@ -36897,21 +36897,21 @@
     <row r="1448">
       <c r="A1448" t="inlineStr">
         <is>
-          <t>ME1049</t>
+          <t>314208</t>
         </is>
       </c>
       <c r="B1448" t="inlineStr">
         <is>
-          <t>TAPA PUSH PULL DORADA ROSCA 24</t>
+          <t>GEMTONE AMBER G001</t>
         </is>
       </c>
       <c r="C1448" t="n">
-        <v>3386</v>
+        <v>73488</v>
       </c>
       <c r="D1448" t="inlineStr"/>
       <c r="E1448" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F1448" t="inlineStr">
@@ -36923,21 +36923,21 @@
     <row r="1449">
       <c r="A1449" t="inlineStr">
         <is>
-          <t>314208</t>
+          <t>ME1049</t>
         </is>
       </c>
       <c r="B1449" t="inlineStr">
         <is>
-          <t>GEMTONE AMBER G001</t>
+          <t>TAPA PUSH PULL DORADA ROSCA 24</t>
         </is>
       </c>
       <c r="C1449" t="n">
-        <v>73488</v>
+        <v>3386</v>
       </c>
       <c r="D1449" t="inlineStr"/>
       <c r="E1449" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1449" t="inlineStr">
@@ -37287,21 +37287,21 @@
     <row r="1463">
       <c r="A1463" t="inlineStr">
         <is>
-          <t>ET0202</t>
+          <t>ME0505</t>
         </is>
       </c>
       <c r="B1463" t="inlineStr">
         <is>
-          <t>ETIQUETA PERFUME CABELLO ARRIESGAD 120ML</t>
+          <t>BALA TRANSPARENTE 120ML</t>
         </is>
       </c>
       <c r="C1463" t="n">
-        <v>140</v>
+        <v>2543</v>
       </c>
       <c r="D1463" t="inlineStr"/>
       <c r="E1463" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1463" t="inlineStr">
@@ -37313,21 +37313,21 @@
     <row r="1464">
       <c r="A1464" t="inlineStr">
         <is>
-          <t>ME0505</t>
+          <t>ET0202</t>
         </is>
       </c>
       <c r="B1464" t="inlineStr">
         <is>
-          <t>BALA TRANSPARENTE 120ML</t>
+          <t>ETIQUETA PERFUME CABELLO ARRIESGAD 120ML</t>
         </is>
       </c>
       <c r="C1464" t="n">
-        <v>2543</v>
+        <v>140</v>
       </c>
       <c r="D1464" t="inlineStr"/>
       <c r="E1464" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1464" t="inlineStr">
@@ -38197,21 +38197,21 @@
     <row r="1498">
       <c r="A1498" t="inlineStr">
         <is>
-          <t>ME1043</t>
+          <t>173501</t>
         </is>
       </c>
       <c r="B1498" t="inlineStr">
         <is>
-          <t>TAPA FLIP TOP DORADA ROSCA 18</t>
+          <t>ULTRAMAR U-200 AZUL</t>
         </is>
       </c>
       <c r="C1498" t="n">
-        <v>4500</v>
+        <v>5979</v>
       </c>
       <c r="D1498" t="inlineStr"/>
       <c r="E1498" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F1498" t="inlineStr">
@@ -38223,16 +38223,16 @@
     <row r="1499">
       <c r="A1499" t="inlineStr">
         <is>
-          <t>ME1044</t>
+          <t>ME1043</t>
         </is>
       </c>
       <c r="B1499" t="inlineStr">
         <is>
-          <t>TAPA FLIP TOP PLATEADA ROSCA 18</t>
+          <t>TAPA FLIP TOP DORADA ROSCA 18</t>
         </is>
       </c>
       <c r="C1499" t="n">
-        <v>39551</v>
+        <v>4500</v>
       </c>
       <c r="D1499" t="inlineStr"/>
       <c r="E1499" t="inlineStr">
@@ -38249,21 +38249,21 @@
     <row r="1500">
       <c r="A1500" t="inlineStr">
         <is>
-          <t>173501</t>
+          <t>ME1044</t>
         </is>
       </c>
       <c r="B1500" t="inlineStr">
         <is>
-          <t>ULTRAMAR U-200 AZUL</t>
+          <t>TAPA FLIP TOP PLATEADA ROSCA 18</t>
         </is>
       </c>
       <c r="C1500" t="n">
-        <v>5979</v>
+        <v>39551</v>
       </c>
       <c r="D1500" t="inlineStr"/>
       <c r="E1500" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1500" t="inlineStr">
@@ -39185,16 +39185,16 @@
     <row r="1536">
       <c r="A1536" t="inlineStr">
         <is>
-          <t>ME1055</t>
+          <t>ME0578</t>
         </is>
       </c>
       <c r="B1536" t="inlineStr">
         <is>
-          <t>TAPA SPRAY VERDE ROSCA 18</t>
+          <t>ENVASE ROJO RUBOR EN CREMA RUBY</t>
         </is>
       </c>
       <c r="C1536" t="n">
-        <v>11362</v>
+        <v>19980</v>
       </c>
       <c r="D1536" t="inlineStr"/>
       <c r="E1536" t="inlineStr">
@@ -39211,16 +39211,16 @@
     <row r="1537">
       <c r="A1537" t="inlineStr">
         <is>
-          <t>ME0511</t>
+          <t>ME0579</t>
         </is>
       </c>
       <c r="B1537" t="inlineStr">
         <is>
-          <t>ENV PEAD KABA B28 500ML</t>
+          <t>ENVASE NARANJA RUBOR EN CREMA SALLY</t>
         </is>
       </c>
       <c r="C1537" t="n">
-        <v>28261</v>
+        <v>19475</v>
       </c>
       <c r="D1537" t="inlineStr"/>
       <c r="E1537" t="inlineStr">
@@ -39237,21 +39237,21 @@
     <row r="1538">
       <c r="A1538" t="inlineStr">
         <is>
-          <t>ET0253</t>
+          <t>ME1067</t>
         </is>
       </c>
       <c r="B1538" t="inlineStr">
         <is>
-          <t>ETIQUETA BRONC DE CHOCOLATE MIEL 45ML</t>
+          <t>TAPA NARANJA RUBOR EN BARRA SALLY</t>
         </is>
       </c>
       <c r="C1538" t="n">
-        <v>22864</v>
+        <v>19440</v>
       </c>
       <c r="D1538" t="inlineStr"/>
       <c r="E1538" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1538" t="inlineStr">
@@ -39263,16 +39263,16 @@
     <row r="1539">
       <c r="A1539" t="inlineStr">
         <is>
-          <t>ME0578</t>
+          <t>ME1055</t>
         </is>
       </c>
       <c r="B1539" t="inlineStr">
         <is>
-          <t>ENVASE ROJO RUBOR EN CREMA RUBY</t>
+          <t>TAPA SPRAY VERDE ROSCA 18</t>
         </is>
       </c>
       <c r="C1539" t="n">
-        <v>19980</v>
+        <v>11362</v>
       </c>
       <c r="D1539" t="inlineStr"/>
       <c r="E1539" t="inlineStr">
@@ -39289,16 +39289,16 @@
     <row r="1540">
       <c r="A1540" t="inlineStr">
         <is>
-          <t>ME0579</t>
+          <t>ME0511</t>
         </is>
       </c>
       <c r="B1540" t="inlineStr">
         <is>
-          <t>ENVASE NARANJA RUBOR EN CREMA SALLY</t>
+          <t>ENV PEAD KABA B28 500ML</t>
         </is>
       </c>
       <c r="C1540" t="n">
-        <v>19475</v>
+        <v>28261</v>
       </c>
       <c r="D1540" t="inlineStr"/>
       <c r="E1540" t="inlineStr">
@@ -39315,21 +39315,21 @@
     <row r="1541">
       <c r="A1541" t="inlineStr">
         <is>
-          <t>ME1067</t>
+          <t>ET0253</t>
         </is>
       </c>
       <c r="B1541" t="inlineStr">
         <is>
-          <t>TAPA NARANJA RUBOR EN BARRA SALLY</t>
+          <t>ETIQUETA BRONC DE CHOCOLATE MIEL 45ML</t>
         </is>
       </c>
       <c r="C1541" t="n">
-        <v>19440</v>
+        <v>22864</v>
       </c>
       <c r="D1541" t="inlineStr"/>
       <c r="E1541" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1541" t="inlineStr">
@@ -39627,16 +39627,16 @@
     <row r="1553">
       <c r="A1553" t="inlineStr">
         <is>
-          <t>ME1028</t>
+          <t>ME0504</t>
         </is>
       </c>
       <c r="B1553" t="inlineStr">
         <is>
-          <t>TAPA CON APLICADOR PUNTA PINCEL</t>
+          <t>BALA NEGRA LARGA 120ML</t>
         </is>
       </c>
       <c r="C1553" t="n">
-        <v>15877</v>
+        <v>9239</v>
       </c>
       <c r="D1553" t="inlineStr"/>
       <c r="E1553" t="inlineStr">
@@ -39653,16 +39653,16 @@
     <row r="1554">
       <c r="A1554" t="inlineStr">
         <is>
-          <t>ME1059</t>
+          <t>ME0507</t>
         </is>
       </c>
       <c r="B1554" t="inlineStr">
         <is>
-          <t>WIPER ( ESCURRIDOR/BARREDOR) NATURAL</t>
+          <t>BALA TRANSPARENTE 30ML</t>
         </is>
       </c>
       <c r="C1554" t="n">
-        <v>30387</v>
+        <v>24300</v>
       </c>
       <c r="D1554" t="inlineStr"/>
       <c r="E1554" t="inlineStr">
@@ -39679,16 +39679,16 @@
     <row r="1555">
       <c r="A1555" t="inlineStr">
         <is>
-          <t>ME0504</t>
+          <t>ME1028</t>
         </is>
       </c>
       <c r="B1555" t="inlineStr">
         <is>
-          <t>BALA NEGRA LARGA 120ML</t>
+          <t>TAPA CON APLICADOR PUNTA PINCEL</t>
         </is>
       </c>
       <c r="C1555" t="n">
-        <v>9239</v>
+        <v>15877</v>
       </c>
       <c r="D1555" t="inlineStr"/>
       <c r="E1555" t="inlineStr">
@@ -39705,16 +39705,16 @@
     <row r="1556">
       <c r="A1556" t="inlineStr">
         <is>
-          <t>ME0507</t>
+          <t>ME1059</t>
         </is>
       </c>
       <c r="B1556" t="inlineStr">
         <is>
-          <t>BALA TRANSPARENTE 30ML</t>
+          <t>WIPER ( ESCURRIDOR/BARREDOR) NATURAL</t>
         </is>
       </c>
       <c r="C1556" t="n">
-        <v>24300</v>
+        <v>30387</v>
       </c>
       <c r="D1556" t="inlineStr"/>
       <c r="E1556" t="inlineStr">
@@ -39913,16 +39913,16 @@
     <row r="1564">
       <c r="A1564" t="inlineStr">
         <is>
-          <t>ME0523</t>
+          <t>ME0542</t>
         </is>
       </c>
       <c r="B1564" t="inlineStr">
         <is>
-          <t>ENVASE PVC COLOR BLANCO POCIMA 6ML</t>
+          <t>TUBO COLAP ANTOBRONCEADORA 120ML V1</t>
         </is>
       </c>
       <c r="C1564" t="n">
-        <v>33606</v>
+        <v>3493</v>
       </c>
       <c r="D1564" t="inlineStr"/>
       <c r="E1564" t="inlineStr">
@@ -39939,16 +39939,16 @@
     <row r="1565">
       <c r="A1565" t="inlineStr">
         <is>
-          <t>ME0542</t>
+          <t>ME0545</t>
         </is>
       </c>
       <c r="B1565" t="inlineStr">
         <is>
-          <t>TUBO COLAP ANTOBRONCEADORA 120ML V1</t>
+          <t>TUBO COLAP EXFOLIANTE CAPILAR 220GR V1</t>
         </is>
       </c>
       <c r="C1565" t="n">
-        <v>3493</v>
+        <v>1909</v>
       </c>
       <c r="D1565" t="inlineStr"/>
       <c r="E1565" t="inlineStr">
@@ -39965,16 +39965,16 @@
     <row r="1566">
       <c r="A1566" t="inlineStr">
         <is>
-          <t>ME0545</t>
+          <t>ME0523</t>
         </is>
       </c>
       <c r="B1566" t="inlineStr">
         <is>
-          <t>TUBO COLAP EXFOLIANTE CAPILAR 220GR V1</t>
+          <t>ENVASE PVC COLOR BLANCO POCIMA 6ML</t>
         </is>
       </c>
       <c r="C1566" t="n">
-        <v>1909</v>
+        <v>33606</v>
       </c>
       <c r="D1566" t="inlineStr"/>
       <c r="E1566" t="inlineStr">
@@ -39991,16 +39991,16 @@
     <row r="1567">
       <c r="A1567" t="inlineStr">
         <is>
-          <t>ME1040</t>
+          <t>ME0513</t>
         </is>
       </c>
       <c r="B1567" t="inlineStr">
         <is>
-          <t>TAPA FLIP TOP 28 MM ROSADO FLAMENCO</t>
+          <t>ENVASE APPLE 28/410 TRANSP P30 M1 300ML</t>
         </is>
       </c>
       <c r="C1567" t="n">
-        <v>17344</v>
+        <v>9838</v>
       </c>
       <c r="D1567" t="inlineStr"/>
       <c r="E1567" t="inlineStr">
@@ -40017,16 +40017,16 @@
     <row r="1568">
       <c r="A1568" t="inlineStr">
         <is>
-          <t>ME0513</t>
+          <t>ME1040</t>
         </is>
       </c>
       <c r="B1568" t="inlineStr">
         <is>
-          <t>ENVASE APPLE 28/410 TRANSP P30 M1 300ML</t>
+          <t>TAPA FLIP TOP 28 MM ROSADO FLAMENCO</t>
         </is>
       </c>
       <c r="C1568" t="n">
-        <v>9838</v>
+        <v>17344</v>
       </c>
       <c r="D1568" t="inlineStr"/>
       <c r="E1568" t="inlineStr">
@@ -41187,16 +41187,16 @@
     <row r="1613">
       <c r="A1613" t="inlineStr">
         <is>
-          <t>ME0519</t>
+          <t>ME0544</t>
         </is>
       </c>
       <c r="B1613" t="inlineStr">
         <is>
-          <t>ENVASE PARA CREMA FACIAL TENSORA</t>
+          <t>TUBO COLAP DERMOACLARANTE 60ML V1</t>
         </is>
       </c>
       <c r="C1613" t="n">
-        <v>10009</v>
+        <v>8240</v>
       </c>
       <c r="D1613" t="inlineStr"/>
       <c r="E1613" t="inlineStr">
@@ -41213,16 +41213,16 @@
     <row r="1614">
       <c r="A1614" t="inlineStr">
         <is>
-          <t>ME1014</t>
+          <t>ME0519</t>
         </is>
       </c>
       <c r="B1614" t="inlineStr">
         <is>
-          <t>SHINE GREEN COLOR PRESS</t>
+          <t>ENVASE PARA CREMA FACIAL TENSORA</t>
         </is>
       </c>
       <c r="C1614" t="n">
-        <v>6885</v>
+        <v>10009</v>
       </c>
       <c r="D1614" t="inlineStr"/>
       <c r="E1614" t="inlineStr">
@@ -41239,16 +41239,16 @@
     <row r="1615">
       <c r="A1615" t="inlineStr">
         <is>
-          <t>ME0544</t>
+          <t>ME1014</t>
         </is>
       </c>
       <c r="B1615" t="inlineStr">
         <is>
-          <t>TUBO COLAP DERMOACLARANTE 60ML V1</t>
+          <t>SHINE GREEN COLOR PRESS</t>
         </is>
       </c>
       <c r="C1615" t="n">
-        <v>8240</v>
+        <v>6885</v>
       </c>
       <c r="D1615" t="inlineStr"/>
       <c r="E1615" t="inlineStr">
@@ -41629,16 +41629,16 @@
     <row r="1630">
       <c r="A1630" t="inlineStr">
         <is>
-          <t>ME1012</t>
+          <t>ME1068</t>
         </is>
       </c>
       <c r="B1630" t="inlineStr">
         <is>
-          <t>BOMBA ENCASQUE DORADA/BRONCEADORES</t>
+          <t>TAPA SPRAY BLANCA R 18/410 (DEPILADOR N)</t>
         </is>
       </c>
       <c r="C1630" t="n">
-        <v>27625</v>
+        <v>257740</v>
       </c>
       <c r="D1630" t="inlineStr"/>
       <c r="E1630" t="inlineStr">
@@ -41655,21 +41655,21 @@
     <row r="1631">
       <c r="A1631" t="inlineStr">
         <is>
-          <t>ET02138</t>
+          <t>ME1012</t>
         </is>
       </c>
       <c r="B1631" t="inlineStr">
         <is>
-          <t>ETIQUETA KERATINA ALISADOR KABA 500 ML</t>
+          <t>BOMBA ENCASQUE DORADA/BRONCEADORES</t>
         </is>
       </c>
       <c r="C1631" t="n">
-        <v>2868</v>
+        <v>27625</v>
       </c>
       <c r="D1631" t="inlineStr"/>
       <c r="E1631" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1631" t="inlineStr">
@@ -41681,16 +41681,16 @@
     <row r="1632">
       <c r="A1632" t="inlineStr">
         <is>
-          <t>ET02139</t>
+          <t>ET02138</t>
         </is>
       </c>
       <c r="B1632" t="inlineStr">
         <is>
-          <t>ETIQUETA KERATINA ALISADOR KABA 250 ML</t>
+          <t>ETIQUETA KERATINA ALISADOR KABA 500 ML</t>
         </is>
       </c>
       <c r="C1632" t="n">
-        <v>1368</v>
+        <v>2868</v>
       </c>
       <c r="D1632" t="inlineStr"/>
       <c r="E1632" t="inlineStr">
@@ -41707,21 +41707,21 @@
     <row r="1633">
       <c r="A1633" t="inlineStr">
         <is>
-          <t>ME1068</t>
+          <t>ET02139</t>
         </is>
       </c>
       <c r="B1633" t="inlineStr">
         <is>
-          <t>TAPA SPRAY BLANCA R 18/410 (DEPILADOR N)</t>
+          <t>ETIQUETA KERATINA ALISADOR KABA 250 ML</t>
         </is>
       </c>
       <c r="C1633" t="n">
-        <v>257740</v>
+        <v>1368</v>
       </c>
       <c r="D1633" t="inlineStr"/>
       <c r="E1633" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1633" t="inlineStr">
@@ -42587,21 +42587,21 @@
     <row r="1667">
       <c r="A1667" t="inlineStr">
         <is>
-          <t>ET0202CA</t>
+          <t>190102</t>
         </is>
       </c>
       <c r="B1667" t="inlineStr">
         <is>
-          <t>ETIQUETA ILUMINADOR GOLD ROSE CARA</t>
+          <t>CARBÓN ACTIVADO</t>
         </is>
       </c>
       <c r="C1667" t="n">
-        <v>3916</v>
+        <v>500</v>
       </c>
       <c r="D1667" t="inlineStr"/>
       <c r="E1667" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F1667" t="inlineStr">
@@ -42613,21 +42613,21 @@
     <row r="1668">
       <c r="A1668" t="inlineStr">
         <is>
-          <t>190102</t>
+          <t>ET0202CA</t>
         </is>
       </c>
       <c r="B1668" t="inlineStr">
         <is>
-          <t>CARBÓN ACTIVADO</t>
+          <t>ETIQUETA ILUMINADOR GOLD ROSE CARA</t>
         </is>
       </c>
       <c r="C1668" t="n">
-        <v>500</v>
+        <v>3916</v>
       </c>
       <c r="D1668" t="inlineStr"/>
       <c r="E1668" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1668" t="inlineStr">
@@ -42691,21 +42691,21 @@
     <row r="1671">
       <c r="A1671" t="inlineStr">
         <is>
-          <t>ETC0160</t>
+          <t>ME0553</t>
         </is>
       </c>
       <c r="B1671" t="inlineStr">
         <is>
-          <t>CAJA RUBOR EN CREMA RUBY</t>
+          <t>TUBO COLAP TTO REVITALIZANTE 230ML V1</t>
         </is>
       </c>
       <c r="C1671" t="n">
-        <v>10536</v>
+        <v>478</v>
       </c>
       <c r="D1671" t="inlineStr"/>
       <c r="E1671" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1671" t="inlineStr">
@@ -42717,16 +42717,16 @@
     <row r="1672">
       <c r="A1672" t="inlineStr">
         <is>
-          <t>ETC0161</t>
+          <t>ETC0160</t>
         </is>
       </c>
       <c r="B1672" t="inlineStr">
         <is>
-          <t>CAJA RUBOR EN CREMA SALLY</t>
+          <t>CAJA RUBOR EN CREMA RUBY</t>
         </is>
       </c>
       <c r="C1672" t="n">
-        <v>10328</v>
+        <v>10536</v>
       </c>
       <c r="D1672" t="inlineStr"/>
       <c r="E1672" t="inlineStr">
@@ -42743,21 +42743,21 @@
     <row r="1673">
       <c r="A1673" t="inlineStr">
         <is>
-          <t>ME0553</t>
+          <t>ETC0161</t>
         </is>
       </c>
       <c r="B1673" t="inlineStr">
         <is>
-          <t>TUBO COLAP TTO REVITALIZANTE 230ML V1</t>
+          <t>CAJA RUBOR EN CREMA SALLY</t>
         </is>
       </c>
       <c r="C1673" t="n">
-        <v>478</v>
+        <v>10328</v>
       </c>
       <c r="D1673" t="inlineStr"/>
       <c r="E1673" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1673" t="inlineStr">
@@ -43289,21 +43289,21 @@
     <row r="1694">
       <c r="A1694" t="inlineStr">
         <is>
-          <t>ETC0173</t>
+          <t>ME0506</t>
         </is>
       </c>
       <c r="B1694" t="inlineStr">
         <is>
-          <t>CAJA TONICO CAPILAR KABA ROSADA 120ML</t>
+          <t>BALA TRANSPARENTE 260/250 ML</t>
         </is>
       </c>
       <c r="C1694" t="n">
-        <v>193</v>
+        <v>9784</v>
       </c>
       <c r="D1694" t="inlineStr"/>
       <c r="E1694" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1694" t="inlineStr">
@@ -43315,21 +43315,21 @@
     <row r="1695">
       <c r="A1695" t="inlineStr">
         <is>
-          <t>ME0506</t>
+          <t>ETC0173</t>
         </is>
       </c>
       <c r="B1695" t="inlineStr">
         <is>
-          <t>BALA TRANSPARENTE 260/250 ML</t>
+          <t>CAJA TONICO CAPILAR KABA ROSADA 120ML</t>
         </is>
       </c>
       <c r="C1695" t="n">
-        <v>9784</v>
+        <v>193</v>
       </c>
       <c r="D1695" t="inlineStr"/>
       <c r="E1695" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1695" t="inlineStr">

</xml_diff>

<commit_message>
Actualizar inventario_operaciones.xlsx (solo-inventario) - 2026-08-18 06:00
</commit_message>
<xml_diff>
--- a/inventario_operaciones.xlsx
+++ b/inventario_operaciones.xlsx
@@ -1207,19 +1207,19 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>R010302</t>
+          <t>K010102</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>TONICO CAPILAR LA RECETA</t>
+          <t>SHAMPO KIDS KABA</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>184</v>
+        <v>120</v>
       </c>
       <c r="D29" t="n">
-        <v>3218.702290076336</v>
+        <v>2141.106870229008</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1235,19 +1235,19 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>K010102</t>
+          <t>R010302</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>SHAMPO KIDS KABA</t>
+          <t>TONICO CAPILAR LA RECETA</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>120</v>
+        <v>184</v>
       </c>
       <c r="D30" t="n">
-        <v>2141.106870229008</v>
+        <v>3218.702290076336</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -8195,19 +8195,19 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>R010302</t>
+          <t>K010102</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>TONICO CAPILAR LA RECETA</t>
+          <t>SHAMPO KIDS KABA</t>
         </is>
       </c>
       <c r="C285" t="n">
-        <v>13873</v>
+        <v>2891</v>
       </c>
       <c r="D285" t="n">
-        <v>3218.702290076336</v>
+        <v>2141.106870229008</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -8223,19 +8223,19 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>K010101</t>
+          <t>R010302</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>SHAMPO DE CEBOLLA KABA</t>
+          <t>TONICO CAPILAR LA RECETA</t>
         </is>
       </c>
       <c r="C286" t="n">
-        <v>176638</v>
+        <v>13873</v>
       </c>
       <c r="D286" t="n">
-        <v>81409.46564885495</v>
+        <v>3218.702290076336</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -8251,19 +8251,19 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>K010102</t>
+          <t>K010101</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>SHAMPO KIDS KABA</t>
+          <t>SHAMPO DE CEBOLLA KABA</t>
         </is>
       </c>
       <c r="C287" t="n">
-        <v>2891</v>
+        <v>176638</v>
       </c>
       <c r="D287" t="n">
-        <v>2141.106870229008</v>
+        <v>81409.46564885495</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -13589,21 +13589,21 @@
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>155301</t>
+          <t>ME1011</t>
         </is>
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>ESTOGEL M</t>
+          <t>LOTIÓN PUMP 28/410 SILVER/WHITE</t>
         </is>
       </c>
       <c r="C486" t="n">
-        <v>100000</v>
+        <v>326790</v>
       </c>
       <c r="D486" t="inlineStr"/>
       <c r="E486" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F486" t="inlineStr">
@@ -13615,21 +13615,21 @@
     <row r="487">
       <c r="A487" t="inlineStr">
         <is>
-          <t>ME1011</t>
+          <t>155301</t>
         </is>
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>LOTIÓN PUMP 28/410 SILVER/WHITE</t>
+          <t>ESTOGEL M</t>
         </is>
       </c>
       <c r="C487" t="n">
-        <v>326790</v>
+        <v>100000</v>
       </c>
       <c r="D487" t="inlineStr"/>
       <c r="E487" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F487" t="inlineStr">
@@ -34791,21 +34791,21 @@
     <row r="1373">
       <c r="A1373" t="inlineStr">
         <is>
-          <t>314208</t>
+          <t>ME1049</t>
         </is>
       </c>
       <c r="B1373" t="inlineStr">
         <is>
-          <t>GEMTONE AMBER G001</t>
+          <t>TAPA PUSH PULL DORADA ROSCA 24</t>
         </is>
       </c>
       <c r="C1373" t="n">
-        <v>73488</v>
+        <v>3386</v>
       </c>
       <c r="D1373" t="inlineStr"/>
       <c r="E1373" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1373" t="inlineStr">
@@ -34817,21 +34817,21 @@
     <row r="1374">
       <c r="A1374" t="inlineStr">
         <is>
-          <t>ME1049</t>
+          <t>314208</t>
         </is>
       </c>
       <c r="B1374" t="inlineStr">
         <is>
-          <t>TAPA PUSH PULL DORADA ROSCA 24</t>
+          <t>GEMTONE AMBER G001</t>
         </is>
       </c>
       <c r="C1374" t="n">
-        <v>3386</v>
+        <v>73488</v>
       </c>
       <c r="D1374" t="inlineStr"/>
       <c r="E1374" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F1374" t="inlineStr">
@@ -35207,21 +35207,21 @@
     <row r="1389">
       <c r="A1389" t="inlineStr">
         <is>
-          <t>ME0505</t>
+          <t>ET0202</t>
         </is>
       </c>
       <c r="B1389" t="inlineStr">
         <is>
-          <t>BALA TRANSPARENTE 120ML</t>
+          <t>ETIQUETA PERFUME CABELLO ARRIESGAD 120ML</t>
         </is>
       </c>
       <c r="C1389" t="n">
-        <v>2543</v>
+        <v>140</v>
       </c>
       <c r="D1389" t="inlineStr"/>
       <c r="E1389" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1389" t="inlineStr">
@@ -35233,21 +35233,21 @@
     <row r="1390">
       <c r="A1390" t="inlineStr">
         <is>
-          <t>ET0202</t>
+          <t>ME0505</t>
         </is>
       </c>
       <c r="B1390" t="inlineStr">
         <is>
-          <t>ETIQUETA PERFUME CABELLO ARRIESGAD 120ML</t>
+          <t>BALA TRANSPARENTE 120ML</t>
         </is>
       </c>
       <c r="C1390" t="n">
-        <v>140</v>
+        <v>2543</v>
       </c>
       <c r="D1390" t="inlineStr"/>
       <c r="E1390" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1390" t="inlineStr">
@@ -36143,21 +36143,21 @@
     <row r="1425">
       <c r="A1425" t="inlineStr">
         <is>
-          <t>173501</t>
+          <t>ME1043</t>
         </is>
       </c>
       <c r="B1425" t="inlineStr">
         <is>
-          <t>ULTRAMAR U-200 AZUL</t>
+          <t>TAPA FLIP TOP DORADA ROSCA 18</t>
         </is>
       </c>
       <c r="C1425" t="n">
-        <v>5310</v>
+        <v>2731</v>
       </c>
       <c r="D1425" t="inlineStr"/>
       <c r="E1425" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1425" t="inlineStr">
@@ -36169,16 +36169,16 @@
     <row r="1426">
       <c r="A1426" t="inlineStr">
         <is>
-          <t>ME1043</t>
+          <t>ME1044</t>
         </is>
       </c>
       <c r="B1426" t="inlineStr">
         <is>
-          <t>TAPA FLIP TOP DORADA ROSCA 18</t>
+          <t>TAPA FLIP TOP PLATEADA ROSCA 18</t>
         </is>
       </c>
       <c r="C1426" t="n">
-        <v>2731</v>
+        <v>39551</v>
       </c>
       <c r="D1426" t="inlineStr"/>
       <c r="E1426" t="inlineStr">
@@ -36195,21 +36195,21 @@
     <row r="1427">
       <c r="A1427" t="inlineStr">
         <is>
-          <t>ME1044</t>
+          <t>173501</t>
         </is>
       </c>
       <c r="B1427" t="inlineStr">
         <is>
-          <t>TAPA FLIP TOP PLATEADA ROSCA 18</t>
+          <t>ULTRAMAR U-200 AZUL</t>
         </is>
       </c>
       <c r="C1427" t="n">
-        <v>39551</v>
+        <v>5310</v>
       </c>
       <c r="D1427" t="inlineStr"/>
       <c r="E1427" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F1427" t="inlineStr">
@@ -37131,16 +37131,16 @@
     <row r="1463">
       <c r="A1463" t="inlineStr">
         <is>
-          <t>ME0578</t>
+          <t>ME0511</t>
         </is>
       </c>
       <c r="B1463" t="inlineStr">
         <is>
-          <t>ENVASE ROJO RUBOR EN CREMA RUBY</t>
+          <t>ENV PEAD KABA B28 500ML</t>
         </is>
       </c>
       <c r="C1463" t="n">
-        <v>19980</v>
+        <v>28261</v>
       </c>
       <c r="D1463" t="inlineStr"/>
       <c r="E1463" t="inlineStr">
@@ -37157,21 +37157,21 @@
     <row r="1464">
       <c r="A1464" t="inlineStr">
         <is>
-          <t>ME0579</t>
+          <t>ET0253</t>
         </is>
       </c>
       <c r="B1464" t="inlineStr">
         <is>
-          <t>ENVASE NARANJA RUBOR EN CREMA SALLY</t>
+          <t>ETIQUETA BRONC DE CHOCOLATE MIEL 45ML</t>
         </is>
       </c>
       <c r="C1464" t="n">
-        <v>19475</v>
+        <v>22864</v>
       </c>
       <c r="D1464" t="inlineStr"/>
       <c r="E1464" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1464" t="inlineStr">
@@ -37183,16 +37183,16 @@
     <row r="1465">
       <c r="A1465" t="inlineStr">
         <is>
-          <t>ME1055</t>
+          <t>ME0578</t>
         </is>
       </c>
       <c r="B1465" t="inlineStr">
         <is>
-          <t>TAPA SPRAY VERDE ROSCA 18</t>
+          <t>ENVASE ROJO RUBOR EN CREMA RUBY</t>
         </is>
       </c>
       <c r="C1465" t="n">
-        <v>11362</v>
+        <v>19980</v>
       </c>
       <c r="D1465" t="inlineStr"/>
       <c r="E1465" t="inlineStr">
@@ -37209,16 +37209,16 @@
     <row r="1466">
       <c r="A1466" t="inlineStr">
         <is>
-          <t>ME1067</t>
+          <t>ME0579</t>
         </is>
       </c>
       <c r="B1466" t="inlineStr">
         <is>
-          <t>TAPA NARANJA RUBOR EN BARRA SALLY</t>
+          <t>ENVASE NARANJA RUBOR EN CREMA SALLY</t>
         </is>
       </c>
       <c r="C1466" t="n">
-        <v>19440</v>
+        <v>19475</v>
       </c>
       <c r="D1466" t="inlineStr"/>
       <c r="E1466" t="inlineStr">
@@ -37235,16 +37235,16 @@
     <row r="1467">
       <c r="A1467" t="inlineStr">
         <is>
-          <t>ME0511</t>
+          <t>ME1055</t>
         </is>
       </c>
       <c r="B1467" t="inlineStr">
         <is>
-          <t>ENV PEAD KABA B28 500ML</t>
+          <t>TAPA SPRAY VERDE ROSCA 18</t>
         </is>
       </c>
       <c r="C1467" t="n">
-        <v>28261</v>
+        <v>11362</v>
       </c>
       <c r="D1467" t="inlineStr"/>
       <c r="E1467" t="inlineStr">
@@ -37261,21 +37261,21 @@
     <row r="1468">
       <c r="A1468" t="inlineStr">
         <is>
-          <t>ET0253</t>
+          <t>ME1067</t>
         </is>
       </c>
       <c r="B1468" t="inlineStr">
         <is>
-          <t>ETIQUETA BRONC DE CHOCOLATE MIEL 45ML</t>
+          <t>TAPA NARANJA RUBOR EN BARRA SALLY</t>
         </is>
       </c>
       <c r="C1468" t="n">
-        <v>22864</v>
+        <v>19440</v>
       </c>
       <c r="D1468" t="inlineStr"/>
       <c r="E1468" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1468" t="inlineStr">
@@ -37755,16 +37755,16 @@
     <row r="1487">
       <c r="A1487" t="inlineStr">
         <is>
-          <t>ME1501</t>
+          <t>ME1039</t>
         </is>
       </c>
       <c r="B1487" t="inlineStr">
         <is>
-          <t>TAPON DE VIDRIO ROSCA 28</t>
+          <t>TAPA FLIP TOP 28 MM MORADO SANGRIA</t>
         </is>
       </c>
       <c r="C1487" t="n">
-        <v>17477</v>
+        <v>39454</v>
       </c>
       <c r="D1487" t="inlineStr"/>
       <c r="E1487" t="inlineStr">
@@ -37781,21 +37781,21 @@
     <row r="1488">
       <c r="A1488" t="inlineStr">
         <is>
-          <t>ME1039</t>
+          <t>ET02124</t>
         </is>
       </c>
       <c r="B1488" t="inlineStr">
         <is>
-          <t>TAPA FLIP TOP 28 MM MORADO SANGRIA</t>
+          <t>ETIQUETA UNGUENTO GRANDE 120GR</t>
         </is>
       </c>
       <c r="C1488" t="n">
-        <v>39454</v>
+        <v>299</v>
       </c>
       <c r="D1488" t="inlineStr"/>
       <c r="E1488" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1488" t="inlineStr">
@@ -37807,21 +37807,21 @@
     <row r="1489">
       <c r="A1489" t="inlineStr">
         <is>
-          <t>ET02124</t>
+          <t>ME1501</t>
         </is>
       </c>
       <c r="B1489" t="inlineStr">
         <is>
-          <t>ETIQUETA UNGUENTO GRANDE 120GR</t>
+          <t>TAPON DE VIDRIO ROSCA 28</t>
         </is>
       </c>
       <c r="C1489" t="n">
-        <v>299</v>
+        <v>17477</v>
       </c>
       <c r="D1489" t="inlineStr"/>
       <c r="E1489" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1489" t="inlineStr">
@@ -39185,21 +39185,21 @@
     <row r="1542">
       <c r="A1542" t="inlineStr">
         <is>
-          <t>ME0543</t>
+          <t>ET0204</t>
         </is>
       </c>
       <c r="B1542" t="inlineStr">
         <is>
-          <t>TUBO COLAP CONTORNO DE OJOS 15ML V1</t>
+          <t>ETIQUETA PERFUME CABELLO SOÑADORA 120ML</t>
         </is>
       </c>
       <c r="C1542" t="n">
-        <v>22670</v>
+        <v>184</v>
       </c>
       <c r="D1542" t="inlineStr"/>
       <c r="E1542" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1542" t="inlineStr">
@@ -39211,21 +39211,21 @@
     <row r="1543">
       <c r="A1543" t="inlineStr">
         <is>
-          <t>ET0204</t>
+          <t>ME0543</t>
         </is>
       </c>
       <c r="B1543" t="inlineStr">
         <is>
-          <t>ETIQUETA PERFUME CABELLO SOÑADORA 120ML</t>
+          <t>TUBO COLAP CONTORNO DE OJOS 15ML V1</t>
         </is>
       </c>
       <c r="C1543" t="n">
-        <v>184</v>
+        <v>22670</v>
       </c>
       <c r="D1543" t="inlineStr"/>
       <c r="E1543" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1543" t="inlineStr">
@@ -39497,16 +39497,16 @@
     <row r="1554">
       <c r="A1554" t="inlineStr">
         <is>
-          <t>ME1068</t>
+          <t>ME1012</t>
         </is>
       </c>
       <c r="B1554" t="inlineStr">
         <is>
-          <t>TAPA SPRAY BLANCA R 18/410 (DEPILADOR N)</t>
+          <t>BOMBA ENCASQUE DORADA/BRONCEADORES</t>
         </is>
       </c>
       <c r="C1554" t="n">
-        <v>257740</v>
+        <v>17600</v>
       </c>
       <c r="D1554" t="inlineStr"/>
       <c r="E1554" t="inlineStr">
@@ -39523,21 +39523,21 @@
     <row r="1555">
       <c r="A1555" t="inlineStr">
         <is>
-          <t>ME1012</t>
+          <t>ET02138</t>
         </is>
       </c>
       <c r="B1555" t="inlineStr">
         <is>
-          <t>BOMBA ENCASQUE DORADA/BRONCEADORES</t>
+          <t>ETIQUETA KERATINA ALISADOR KABA 500 ML</t>
         </is>
       </c>
       <c r="C1555" t="n">
-        <v>17600</v>
+        <v>2868</v>
       </c>
       <c r="D1555" t="inlineStr"/>
       <c r="E1555" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1555" t="inlineStr">
@@ -39549,16 +39549,16 @@
     <row r="1556">
       <c r="A1556" t="inlineStr">
         <is>
-          <t>ET02138</t>
+          <t>ET02139</t>
         </is>
       </c>
       <c r="B1556" t="inlineStr">
         <is>
-          <t>ETIQUETA KERATINA ALISADOR KABA 500 ML</t>
+          <t>ETIQUETA KERATINA ALISADOR KABA 250 ML</t>
         </is>
       </c>
       <c r="C1556" t="n">
-        <v>2868</v>
+        <v>1368</v>
       </c>
       <c r="D1556" t="inlineStr"/>
       <c r="E1556" t="inlineStr">
@@ -39575,21 +39575,21 @@
     <row r="1557">
       <c r="A1557" t="inlineStr">
         <is>
-          <t>ET02139</t>
+          <t>ME1068</t>
         </is>
       </c>
       <c r="B1557" t="inlineStr">
         <is>
-          <t>ETIQUETA KERATINA ALISADOR KABA 250 ML</t>
+          <t>TAPA SPRAY BLANCA R 18/410 (DEPILADOR N)</t>
         </is>
       </c>
       <c r="C1557" t="n">
-        <v>1368</v>
+        <v>257740</v>
       </c>
       <c r="D1557" t="inlineStr"/>
       <c r="E1557" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1557" t="inlineStr">
@@ -40065,21 +40065,21 @@
     <row r="1576">
       <c r="A1576" t="inlineStr">
         <is>
-          <t>314202</t>
+          <t>ME0527</t>
         </is>
       </c>
       <c r="B1576" t="inlineStr">
         <is>
-          <t>CLOISONNE ROUGE FLAMBE 440X</t>
+          <t>ENVASE VIDRIO ROSADO MARCADO 30ML</t>
         </is>
       </c>
       <c r="C1576" t="n">
-        <v>6266</v>
+        <v>46</v>
       </c>
       <c r="D1576" t="inlineStr"/>
       <c r="E1576" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1576" t="inlineStr">
@@ -40091,21 +40091,21 @@
     <row r="1577">
       <c r="A1577" t="inlineStr">
         <is>
-          <t>ME0527</t>
+          <t>314202</t>
         </is>
       </c>
       <c r="B1577" t="inlineStr">
         <is>
-          <t>ENVASE VIDRIO ROSADO MARCADO 30ML</t>
+          <t>CLOISONNE ROUGE FLAMBE 440X</t>
         </is>
       </c>
       <c r="C1577" t="n">
-        <v>46</v>
+        <v>6266</v>
       </c>
       <c r="D1577" t="inlineStr"/>
       <c r="E1577" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F1577" t="inlineStr">
@@ -40403,21 +40403,21 @@
     <row r="1589">
       <c r="A1589" t="inlineStr">
         <is>
-          <t>190102</t>
+          <t>ET0202CA</t>
         </is>
       </c>
       <c r="B1589" t="inlineStr">
         <is>
-          <t>CARBÓN ACTIVADO</t>
+          <t>ETIQUETA ILUMINADOR GOLD ROSE CARA</t>
         </is>
       </c>
       <c r="C1589" t="n">
-        <v>500</v>
+        <v>3916</v>
       </c>
       <c r="D1589" t="inlineStr"/>
       <c r="E1589" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1589" t="inlineStr">
@@ -40429,21 +40429,21 @@
     <row r="1590">
       <c r="A1590" t="inlineStr">
         <is>
-          <t>ET0202CA</t>
+          <t>190102</t>
         </is>
       </c>
       <c r="B1590" t="inlineStr">
         <is>
-          <t>ETIQUETA ILUMINADOR GOLD ROSE CARA</t>
+          <t>CARBÓN ACTIVADO</t>
         </is>
       </c>
       <c r="C1590" t="n">
-        <v>3916</v>
+        <v>500</v>
       </c>
       <c r="D1590" t="inlineStr"/>
       <c r="E1590" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F1590" t="inlineStr">
@@ -40507,21 +40507,21 @@
     <row r="1593">
       <c r="A1593" t="inlineStr">
         <is>
-          <t>ME0553</t>
+          <t>ETC0160</t>
         </is>
       </c>
       <c r="B1593" t="inlineStr">
         <is>
-          <t>TUBO COLAP TTO REVITALIZANTE 230ML V1</t>
+          <t>CAJA RUBOR EN CREMA RUBY</t>
         </is>
       </c>
       <c r="C1593" t="n">
-        <v>478</v>
+        <v>10536</v>
       </c>
       <c r="D1593" t="inlineStr"/>
       <c r="E1593" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1593" t="inlineStr">
@@ -40533,16 +40533,16 @@
     <row r="1594">
       <c r="A1594" t="inlineStr">
         <is>
-          <t>ETC0160</t>
+          <t>ETC0161</t>
         </is>
       </c>
       <c r="B1594" t="inlineStr">
         <is>
-          <t>CAJA RUBOR EN CREMA RUBY</t>
+          <t>CAJA RUBOR EN CREMA SALLY</t>
         </is>
       </c>
       <c r="C1594" t="n">
-        <v>10536</v>
+        <v>10328</v>
       </c>
       <c r="D1594" t="inlineStr"/>
       <c r="E1594" t="inlineStr">
@@ -40559,21 +40559,21 @@
     <row r="1595">
       <c r="A1595" t="inlineStr">
         <is>
-          <t>ETC0161</t>
+          <t>ME0553</t>
         </is>
       </c>
       <c r="B1595" t="inlineStr">
         <is>
-          <t>CAJA RUBOR EN CREMA SALLY</t>
+          <t>TUBO COLAP TTO REVITALIZANTE 230ML V1</t>
         </is>
       </c>
       <c r="C1595" t="n">
-        <v>10328</v>
+        <v>478</v>
       </c>
       <c r="D1595" t="inlineStr"/>
       <c r="E1595" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1595" t="inlineStr">
@@ -41105,21 +41105,21 @@
     <row r="1616">
       <c r="A1616" t="inlineStr">
         <is>
-          <t>ME0506</t>
+          <t>ETC0173</t>
         </is>
       </c>
       <c r="B1616" t="inlineStr">
         <is>
-          <t>BALA TRANSPARENTE 260/250 ML</t>
+          <t>CAJA TONICO CAPILAR KABA ROSADA 120ML</t>
         </is>
       </c>
       <c r="C1616" t="n">
-        <v>4464</v>
+        <v>193</v>
       </c>
       <c r="D1616" t="inlineStr"/>
       <c r="E1616" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1616" t="inlineStr">
@@ -41131,21 +41131,21 @@
     <row r="1617">
       <c r="A1617" t="inlineStr">
         <is>
-          <t>ETC0173</t>
+          <t>ME0506</t>
         </is>
       </c>
       <c r="B1617" t="inlineStr">
         <is>
-          <t>CAJA TONICO CAPILAR KABA ROSADA 120ML</t>
+          <t>BALA TRANSPARENTE 260/250 ML</t>
         </is>
       </c>
       <c r="C1617" t="n">
-        <v>193</v>
+        <v>4464</v>
       </c>
       <c r="D1617" t="inlineStr"/>
       <c r="E1617" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1617" t="inlineStr">
@@ -41261,16 +41261,16 @@
     <row r="1622">
       <c r="A1622" t="inlineStr">
         <is>
-          <t>ME0515VG</t>
+          <t>ME1001VG</t>
         </is>
       </c>
       <c r="B1622" t="inlineStr">
         <is>
-          <t>ENVASE CAPSULA BRONCEADOR VIVIANA GRONDO</t>
+          <t>TAPA BRONCEADOR R/24 VIVIANA GRONDONA</t>
         </is>
       </c>
       <c r="C1622" t="n">
-        <v>11568</v>
+        <v>12219</v>
       </c>
       <c r="D1622" t="inlineStr"/>
       <c r="E1622" t="inlineStr">
@@ -41287,16 +41287,16 @@
     <row r="1623">
       <c r="A1623" t="inlineStr">
         <is>
-          <t>ME1001VG</t>
+          <t>ME0533VG</t>
         </is>
       </c>
       <c r="B1623" t="inlineStr">
         <is>
-          <t>TAPA BRONCEADOR R/24 VIVIANA GRONDONA</t>
+          <t>ENVASE Y TAPA APLICADOR VIVIANA GRONDONA</t>
         </is>
       </c>
       <c r="C1623" t="n">
-        <v>12219</v>
+        <v>11568</v>
       </c>
       <c r="D1623" t="inlineStr"/>
       <c r="E1623" t="inlineStr">
@@ -41313,12 +41313,12 @@
     <row r="1624">
       <c r="A1624" t="inlineStr">
         <is>
-          <t>ME0533VG</t>
+          <t>ME0515VG</t>
         </is>
       </c>
       <c r="B1624" t="inlineStr">
         <is>
-          <t>ENVASE Y TAPA APLICADOR VIVIANA GRONDONA</t>
+          <t>ENVASE CAPSULA BRONCEADOR VIVIANA GRONDO</t>
         </is>
       </c>
       <c r="C1624" t="n">
@@ -45285,21 +45285,21 @@
     <row r="1773">
       <c r="A1773" t="inlineStr">
         <is>
-          <t>144301</t>
+          <t>ET0204VG</t>
         </is>
       </c>
       <c r="B1773" t="inlineStr">
         <is>
-          <t>ALCOHOL CETOESTEARÍLICO 30/70</t>
+          <t>ETIQUETA LIP GLOSS VIVIANA GRONDONA D2</t>
         </is>
       </c>
       <c r="C1773" t="n">
-        <v>96090</v>
+        <v>2500</v>
       </c>
       <c r="D1773" t="inlineStr"/>
       <c r="E1773" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1773" t="inlineStr">
@@ -45311,12 +45311,12 @@
     <row r="1774">
       <c r="A1774" t="inlineStr">
         <is>
-          <t>ET0204VG</t>
+          <t>ET0203VG</t>
         </is>
       </c>
       <c r="B1774" t="inlineStr">
         <is>
-          <t>ETIQUETA LIP GLOSS VIVIANA GRONDONA D2</t>
+          <t>ETIQUETA LIP GLOSS VIVIANA GRONDONA D1</t>
         </is>
       </c>
       <c r="C1774" t="n">
@@ -45337,21 +45337,21 @@
     <row r="1775">
       <c r="A1775" t="inlineStr">
         <is>
-          <t>ET0203VG</t>
+          <t>144301</t>
         </is>
       </c>
       <c r="B1775" t="inlineStr">
         <is>
-          <t>ETIQUETA LIP GLOSS VIVIANA GRONDONA D1</t>
+          <t>ALCOHOL CETOESTEARÍLICO 30/70</t>
         </is>
       </c>
       <c r="C1775" t="n">
-        <v>2500</v>
+        <v>96090</v>
       </c>
       <c r="D1775" t="inlineStr"/>
       <c r="E1775" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F1775" t="inlineStr">
@@ -46767,16 +46767,16 @@
     <row r="1830">
       <c r="A1830" t="inlineStr">
         <is>
-          <t>ME0544</t>
+          <t>ME0572</t>
         </is>
       </c>
       <c r="B1830" t="inlineStr">
         <is>
-          <t>TUBO COLAP DERMOACLARANTE 60ML V1</t>
+          <t>COLAPSIBLE AZUL CREMA CORPORAL ACLARANTE</t>
         </is>
       </c>
       <c r="C1830" t="n">
-        <v>815</v>
+        <v>6750</v>
       </c>
       <c r="D1830" t="inlineStr"/>
       <c r="E1830" t="inlineStr">
@@ -46793,16 +46793,16 @@
     <row r="1831">
       <c r="A1831" t="inlineStr">
         <is>
-          <t>ME0572</t>
+          <t>ME0544</t>
         </is>
       </c>
       <c r="B1831" t="inlineStr">
         <is>
-          <t>COLAPSIBLE AZUL CREMA CORPORAL ACLARANTE</t>
+          <t>TUBO COLAP DERMOACLARANTE 60ML V1</t>
         </is>
       </c>
       <c r="C1831" t="n">
-        <v>6750</v>
+        <v>815</v>
       </c>
       <c r="D1831" t="inlineStr"/>
       <c r="E1831" t="inlineStr">

</xml_diff>

<commit_message>
Actualizar inventario_operaciones.xlsx - 2026-08-18 06:15
</commit_message>
<xml_diff>
--- a/inventario_operaciones.xlsx
+++ b/inventario_operaciones.xlsx
@@ -572,7 +572,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>500</v>
+        <v>496</v>
       </c>
       <c r="D6" t="n">
         <v>423.8931297709924</v>
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>622</v>
+        <v>619</v>
       </c>
       <c r="D8" t="n">
         <v>171.412213740458</v>
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="D9" t="n">
         <v>531.7557251908397</v>
@@ -796,7 +796,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="D14" t="n">
         <v>1100.954198473282</v>
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>-46</v>
+        <v>-54</v>
       </c>
       <c r="D15" t="n">
         <v>1163.473282442748</v>
@@ -992,7 +992,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>324</v>
+        <v>316</v>
       </c>
       <c r="D21" t="n">
         <v>1723.396946564885</v>
@@ -1020,7 +1020,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1076</v>
+        <v>1072</v>
       </c>
       <c r="D22" t="n">
         <v>1647.137404580153</v>
@@ -1048,7 +1048,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>-1572</v>
+        <v>-1587</v>
       </c>
       <c r="D23" t="n">
         <v>23981.2213740458</v>
@@ -1104,7 +1104,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D25" t="n">
         <v>21.87022900763359</v>
@@ -1244,7 +1244,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="D30" t="n">
         <v>3218.702290076336</v>
@@ -1300,7 +1300,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="D32" t="n">
         <v>33819.04580152671</v>
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="D35" t="n">
         <v>8401.603053435116</v>
@@ -1468,7 +1468,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="D38" t="n">
         <v>574.0076335877862</v>
@@ -1552,7 +1552,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>101</v>
+        <v>131</v>
       </c>
       <c r="D41" t="n">
         <v>1825.763358778626</v>
@@ -1832,7 +1832,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>778</v>
+        <v>768</v>
       </c>
       <c r="D51" t="n">
         <v>162.824427480916</v>
@@ -1860,7 +1860,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>642</v>
+        <v>638</v>
       </c>
       <c r="D52" t="n">
         <v>101.6793893129771</v>
@@ -2248,7 +2248,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>673</v>
+        <v>667</v>
       </c>
       <c r="D66" t="n">
         <v>15285.91603053435</v>
@@ -2496,7 +2496,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D75" t="n">
         <v>4484.885496183206</v>
@@ -2552,7 +2552,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1174</v>
+        <v>1170</v>
       </c>
       <c r="D77" t="n">
         <v>11863.1679389313</v>
@@ -2688,7 +2688,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="D82" t="n">
         <v>239.0839694656489</v>
@@ -3070,7 +3070,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D96" t="n">
         <v>8045.038167938931</v>
@@ -3178,7 +3178,7 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D100" t="n">
         <v>6729.73282442748</v>
@@ -3262,7 +3262,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D103" t="n">
         <v>230.7251908396946</v>
@@ -3372,7 +3372,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="D107" t="n">
         <v>1616.908396946565</v>
@@ -3456,7 +3456,7 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D110" t="n">
         <v>4274.312977099236</v>
@@ -3652,7 +3652,7 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D117" t="n">
         <v>324.2748091603053</v>
@@ -3788,7 +3788,7 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D122" t="n">
         <v>87.25190839694656</v>
@@ -3984,7 +3984,7 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D129" t="n">
         <v>260.9541984732824</v>
@@ -4012,7 +4012,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="D130" t="n">
         <v>196.8320610687023</v>
@@ -4176,7 +4176,7 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>-807</v>
+        <v>-823</v>
       </c>
       <c r="D136" t="n">
         <v>38473.96946564886</v>
@@ -4204,7 +4204,7 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D137" t="n">
         <v>408.7786259541984</v>
@@ -4336,7 +4336,7 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>825</v>
+        <v>821</v>
       </c>
       <c r="D142" t="n">
         <v>5048.244274809161</v>
@@ -4364,7 +4364,7 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="D143" t="n">
         <v>98.58778625954199</v>
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D148" t="n">
         <v>383.3587786259542</v>
@@ -4558,7 +4558,7 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D150" t="n">
         <v>118.5114503816794</v>
@@ -4586,7 +4586,7 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D151" t="n">
         <v>82.32824427480917</v>
@@ -4696,7 +4696,7 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="D155" t="n">
         <v>164.7709923664122</v>
@@ -4884,7 +4884,7 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="D162" t="n">
         <v>722.9770992366413</v>
@@ -4968,7 +4968,7 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="D165" t="n">
         <v>64.58015267175571</v>
@@ -5024,7 +5024,7 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D167" t="inlineStr"/>
       <c r="E167" t="inlineStr">
@@ -5774,7 +5774,7 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="D195" t="n">
         <v>39274.69465648855</v>
@@ -5802,7 +5802,7 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>2259</v>
+        <v>2256</v>
       </c>
       <c r="D196" t="n">
         <v>32942.74809160305</v>
@@ -13589,21 +13589,21 @@
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>ME1011</t>
+          <t>155301</t>
         </is>
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>LOTIÓN PUMP 28/410 SILVER/WHITE</t>
+          <t>ESTOGEL M</t>
         </is>
       </c>
       <c r="C486" t="n">
-        <v>326790</v>
+        <v>100000</v>
       </c>
       <c r="D486" t="inlineStr"/>
       <c r="E486" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F486" t="inlineStr">
@@ -13615,21 +13615,21 @@
     <row r="487">
       <c r="A487" t="inlineStr">
         <is>
-          <t>155301</t>
+          <t>ME1011</t>
         </is>
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>ESTOGEL M</t>
+          <t>LOTIÓN PUMP 28/410 SILVER/WHITE</t>
         </is>
       </c>
       <c r="C487" t="n">
-        <v>100000</v>
+        <v>326790</v>
       </c>
       <c r="D487" t="inlineStr"/>
       <c r="E487" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F487" t="inlineStr">
@@ -25192,7 +25192,7 @@
         </is>
       </c>
       <c r="C987" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D987" t="inlineStr"/>
       <c r="E987" t="inlineStr"/>
@@ -34791,21 +34791,21 @@
     <row r="1373">
       <c r="A1373" t="inlineStr">
         <is>
-          <t>ME1049</t>
+          <t>314208</t>
         </is>
       </c>
       <c r="B1373" t="inlineStr">
         <is>
-          <t>TAPA PUSH PULL DORADA ROSCA 24</t>
+          <t>GEMTONE AMBER G001</t>
         </is>
       </c>
       <c r="C1373" t="n">
-        <v>3386</v>
+        <v>73488</v>
       </c>
       <c r="D1373" t="inlineStr"/>
       <c r="E1373" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F1373" t="inlineStr">
@@ -34817,21 +34817,21 @@
     <row r="1374">
       <c r="A1374" t="inlineStr">
         <is>
-          <t>314208</t>
+          <t>ME1049</t>
         </is>
       </c>
       <c r="B1374" t="inlineStr">
         <is>
-          <t>GEMTONE AMBER G001</t>
+          <t>TAPA PUSH PULL DORADA ROSCA 24</t>
         </is>
       </c>
       <c r="C1374" t="n">
-        <v>73488</v>
+        <v>3386</v>
       </c>
       <c r="D1374" t="inlineStr"/>
       <c r="E1374" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1374" t="inlineStr">
@@ -35207,21 +35207,21 @@
     <row r="1389">
       <c r="A1389" t="inlineStr">
         <is>
-          <t>ET0202</t>
+          <t>ME0505</t>
         </is>
       </c>
       <c r="B1389" t="inlineStr">
         <is>
-          <t>ETIQUETA PERFUME CABELLO ARRIESGAD 120ML</t>
+          <t>BALA TRANSPARENTE 120ML</t>
         </is>
       </c>
       <c r="C1389" t="n">
-        <v>140</v>
+        <v>2543</v>
       </c>
       <c r="D1389" t="inlineStr"/>
       <c r="E1389" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1389" t="inlineStr">
@@ -35233,21 +35233,21 @@
     <row r="1390">
       <c r="A1390" t="inlineStr">
         <is>
-          <t>ME0505</t>
+          <t>ET0202</t>
         </is>
       </c>
       <c r="B1390" t="inlineStr">
         <is>
-          <t>BALA TRANSPARENTE 120ML</t>
+          <t>ETIQUETA PERFUME CABELLO ARRIESGAD 120ML</t>
         </is>
       </c>
       <c r="C1390" t="n">
-        <v>2543</v>
+        <v>140</v>
       </c>
       <c r="D1390" t="inlineStr"/>
       <c r="E1390" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1390" t="inlineStr">
@@ -36143,21 +36143,21 @@
     <row r="1425">
       <c r="A1425" t="inlineStr">
         <is>
-          <t>ME1043</t>
+          <t>173501</t>
         </is>
       </c>
       <c r="B1425" t="inlineStr">
         <is>
-          <t>TAPA FLIP TOP DORADA ROSCA 18</t>
+          <t>ULTRAMAR U-200 AZUL</t>
         </is>
       </c>
       <c r="C1425" t="n">
-        <v>2731</v>
+        <v>5310</v>
       </c>
       <c r="D1425" t="inlineStr"/>
       <c r="E1425" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F1425" t="inlineStr">
@@ -36169,16 +36169,16 @@
     <row r="1426">
       <c r="A1426" t="inlineStr">
         <is>
-          <t>ME1044</t>
+          <t>ME1043</t>
         </is>
       </c>
       <c r="B1426" t="inlineStr">
         <is>
-          <t>TAPA FLIP TOP PLATEADA ROSCA 18</t>
+          <t>TAPA FLIP TOP DORADA ROSCA 18</t>
         </is>
       </c>
       <c r="C1426" t="n">
-        <v>39551</v>
+        <v>2731</v>
       </c>
       <c r="D1426" t="inlineStr"/>
       <c r="E1426" t="inlineStr">
@@ -36195,21 +36195,21 @@
     <row r="1427">
       <c r="A1427" t="inlineStr">
         <is>
-          <t>173501</t>
+          <t>ME1044</t>
         </is>
       </c>
       <c r="B1427" t="inlineStr">
         <is>
-          <t>ULTRAMAR U-200 AZUL</t>
+          <t>TAPA FLIP TOP PLATEADA ROSCA 18</t>
         </is>
       </c>
       <c r="C1427" t="n">
-        <v>5310</v>
+        <v>39551</v>
       </c>
       <c r="D1427" t="inlineStr"/>
       <c r="E1427" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1427" t="inlineStr">
@@ -37131,16 +37131,16 @@
     <row r="1463">
       <c r="A1463" t="inlineStr">
         <is>
-          <t>ME0511</t>
+          <t>ME0578</t>
         </is>
       </c>
       <c r="B1463" t="inlineStr">
         <is>
-          <t>ENV PEAD KABA B28 500ML</t>
+          <t>ENVASE ROJO RUBOR EN CREMA RUBY</t>
         </is>
       </c>
       <c r="C1463" t="n">
-        <v>28261</v>
+        <v>19980</v>
       </c>
       <c r="D1463" t="inlineStr"/>
       <c r="E1463" t="inlineStr">
@@ -37157,21 +37157,21 @@
     <row r="1464">
       <c r="A1464" t="inlineStr">
         <is>
-          <t>ET0253</t>
+          <t>ME0579</t>
         </is>
       </c>
       <c r="B1464" t="inlineStr">
         <is>
-          <t>ETIQUETA BRONC DE CHOCOLATE MIEL 45ML</t>
+          <t>ENVASE NARANJA RUBOR EN CREMA SALLY</t>
         </is>
       </c>
       <c r="C1464" t="n">
-        <v>22864</v>
+        <v>19475</v>
       </c>
       <c r="D1464" t="inlineStr"/>
       <c r="E1464" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1464" t="inlineStr">
@@ -37183,16 +37183,16 @@
     <row r="1465">
       <c r="A1465" t="inlineStr">
         <is>
-          <t>ME0578</t>
+          <t>ME1055</t>
         </is>
       </c>
       <c r="B1465" t="inlineStr">
         <is>
-          <t>ENVASE ROJO RUBOR EN CREMA RUBY</t>
+          <t>TAPA SPRAY VERDE ROSCA 18</t>
         </is>
       </c>
       <c r="C1465" t="n">
-        <v>19980</v>
+        <v>11362</v>
       </c>
       <c r="D1465" t="inlineStr"/>
       <c r="E1465" t="inlineStr">
@@ -37209,16 +37209,16 @@
     <row r="1466">
       <c r="A1466" t="inlineStr">
         <is>
-          <t>ME0579</t>
+          <t>ME1067</t>
         </is>
       </c>
       <c r="B1466" t="inlineStr">
         <is>
-          <t>ENVASE NARANJA RUBOR EN CREMA SALLY</t>
+          <t>TAPA NARANJA RUBOR EN BARRA SALLY</t>
         </is>
       </c>
       <c r="C1466" t="n">
-        <v>19475</v>
+        <v>19440</v>
       </c>
       <c r="D1466" t="inlineStr"/>
       <c r="E1466" t="inlineStr">
@@ -37235,16 +37235,16 @@
     <row r="1467">
       <c r="A1467" t="inlineStr">
         <is>
-          <t>ME1055</t>
+          <t>ME0511</t>
         </is>
       </c>
       <c r="B1467" t="inlineStr">
         <is>
-          <t>TAPA SPRAY VERDE ROSCA 18</t>
+          <t>ENV PEAD KABA B28 500ML</t>
         </is>
       </c>
       <c r="C1467" t="n">
-        <v>11362</v>
+        <v>28261</v>
       </c>
       <c r="D1467" t="inlineStr"/>
       <c r="E1467" t="inlineStr">
@@ -37261,21 +37261,21 @@
     <row r="1468">
       <c r="A1468" t="inlineStr">
         <is>
-          <t>ME1067</t>
+          <t>ET0253</t>
         </is>
       </c>
       <c r="B1468" t="inlineStr">
         <is>
-          <t>TAPA NARANJA RUBOR EN BARRA SALLY</t>
+          <t>ETIQUETA BRONC DE CHOCOLATE MIEL 45ML</t>
         </is>
       </c>
       <c r="C1468" t="n">
-        <v>19440</v>
+        <v>22864</v>
       </c>
       <c r="D1468" t="inlineStr"/>
       <c r="E1468" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1468" t="inlineStr">
@@ -37755,16 +37755,16 @@
     <row r="1487">
       <c r="A1487" t="inlineStr">
         <is>
-          <t>ME1039</t>
+          <t>ME1501</t>
         </is>
       </c>
       <c r="B1487" t="inlineStr">
         <is>
-          <t>TAPA FLIP TOP 28 MM MORADO SANGRIA</t>
+          <t>TAPON DE VIDRIO ROSCA 28</t>
         </is>
       </c>
       <c r="C1487" t="n">
-        <v>39454</v>
+        <v>17477</v>
       </c>
       <c r="D1487" t="inlineStr"/>
       <c r="E1487" t="inlineStr">
@@ -37781,21 +37781,21 @@
     <row r="1488">
       <c r="A1488" t="inlineStr">
         <is>
-          <t>ET02124</t>
+          <t>ME1039</t>
         </is>
       </c>
       <c r="B1488" t="inlineStr">
         <is>
-          <t>ETIQUETA UNGUENTO GRANDE 120GR</t>
+          <t>TAPA FLIP TOP 28 MM MORADO SANGRIA</t>
         </is>
       </c>
       <c r="C1488" t="n">
-        <v>299</v>
+        <v>39454</v>
       </c>
       <c r="D1488" t="inlineStr"/>
       <c r="E1488" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1488" t="inlineStr">
@@ -37807,21 +37807,21 @@
     <row r="1489">
       <c r="A1489" t="inlineStr">
         <is>
-          <t>ME1501</t>
+          <t>ET02124</t>
         </is>
       </c>
       <c r="B1489" t="inlineStr">
         <is>
-          <t>TAPON DE VIDRIO ROSCA 28</t>
+          <t>ETIQUETA UNGUENTO GRANDE 120GR</t>
         </is>
       </c>
       <c r="C1489" t="n">
-        <v>17477</v>
+        <v>299</v>
       </c>
       <c r="D1489" t="inlineStr"/>
       <c r="E1489" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1489" t="inlineStr">
@@ -39185,21 +39185,21 @@
     <row r="1542">
       <c r="A1542" t="inlineStr">
         <is>
-          <t>ET0204</t>
+          <t>ME0543</t>
         </is>
       </c>
       <c r="B1542" t="inlineStr">
         <is>
-          <t>ETIQUETA PERFUME CABELLO SOÑADORA 120ML</t>
+          <t>TUBO COLAP CONTORNO DE OJOS 15ML V1</t>
         </is>
       </c>
       <c r="C1542" t="n">
-        <v>184</v>
+        <v>22670</v>
       </c>
       <c r="D1542" t="inlineStr"/>
       <c r="E1542" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1542" t="inlineStr">
@@ -39211,21 +39211,21 @@
     <row r="1543">
       <c r="A1543" t="inlineStr">
         <is>
-          <t>ME0543</t>
+          <t>ET0204</t>
         </is>
       </c>
       <c r="B1543" t="inlineStr">
         <is>
-          <t>TUBO COLAP CONTORNO DE OJOS 15ML V1</t>
+          <t>ETIQUETA PERFUME CABELLO SOÑADORA 120ML</t>
         </is>
       </c>
       <c r="C1543" t="n">
-        <v>22670</v>
+        <v>184</v>
       </c>
       <c r="D1543" t="inlineStr"/>
       <c r="E1543" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1543" t="inlineStr">
@@ -39497,16 +39497,16 @@
     <row r="1554">
       <c r="A1554" t="inlineStr">
         <is>
-          <t>ME1012</t>
+          <t>ME1068</t>
         </is>
       </c>
       <c r="B1554" t="inlineStr">
         <is>
-          <t>BOMBA ENCASQUE DORADA/BRONCEADORES</t>
+          <t>TAPA SPRAY BLANCA R 18/410 (DEPILADOR N)</t>
         </is>
       </c>
       <c r="C1554" t="n">
-        <v>17600</v>
+        <v>257740</v>
       </c>
       <c r="D1554" t="inlineStr"/>
       <c r="E1554" t="inlineStr">
@@ -39523,21 +39523,21 @@
     <row r="1555">
       <c r="A1555" t="inlineStr">
         <is>
-          <t>ET02138</t>
+          <t>ME1012</t>
         </is>
       </c>
       <c r="B1555" t="inlineStr">
         <is>
-          <t>ETIQUETA KERATINA ALISADOR KABA 500 ML</t>
+          <t>BOMBA ENCASQUE DORADA/BRONCEADORES</t>
         </is>
       </c>
       <c r="C1555" t="n">
-        <v>2868</v>
+        <v>17600</v>
       </c>
       <c r="D1555" t="inlineStr"/>
       <c r="E1555" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1555" t="inlineStr">
@@ -39549,16 +39549,16 @@
     <row r="1556">
       <c r="A1556" t="inlineStr">
         <is>
-          <t>ET02139</t>
+          <t>ET02138</t>
         </is>
       </c>
       <c r="B1556" t="inlineStr">
         <is>
-          <t>ETIQUETA KERATINA ALISADOR KABA 250 ML</t>
+          <t>ETIQUETA KERATINA ALISADOR KABA 500 ML</t>
         </is>
       </c>
       <c r="C1556" t="n">
-        <v>1368</v>
+        <v>2868</v>
       </c>
       <c r="D1556" t="inlineStr"/>
       <c r="E1556" t="inlineStr">
@@ -39575,21 +39575,21 @@
     <row r="1557">
       <c r="A1557" t="inlineStr">
         <is>
-          <t>ME1068</t>
+          <t>ET02139</t>
         </is>
       </c>
       <c r="B1557" t="inlineStr">
         <is>
-          <t>TAPA SPRAY BLANCA R 18/410 (DEPILADOR N)</t>
+          <t>ETIQUETA KERATINA ALISADOR KABA 250 ML</t>
         </is>
       </c>
       <c r="C1557" t="n">
-        <v>257740</v>
+        <v>1368</v>
       </c>
       <c r="D1557" t="inlineStr"/>
       <c r="E1557" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1557" t="inlineStr">
@@ -40065,21 +40065,21 @@
     <row r="1576">
       <c r="A1576" t="inlineStr">
         <is>
-          <t>ME0527</t>
+          <t>314202</t>
         </is>
       </c>
       <c r="B1576" t="inlineStr">
         <is>
-          <t>ENVASE VIDRIO ROSADO MARCADO 30ML</t>
+          <t>CLOISONNE ROUGE FLAMBE 440X</t>
         </is>
       </c>
       <c r="C1576" t="n">
-        <v>46</v>
+        <v>6266</v>
       </c>
       <c r="D1576" t="inlineStr"/>
       <c r="E1576" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F1576" t="inlineStr">
@@ -40091,21 +40091,21 @@
     <row r="1577">
       <c r="A1577" t="inlineStr">
         <is>
-          <t>314202</t>
+          <t>ME0527</t>
         </is>
       </c>
       <c r="B1577" t="inlineStr">
         <is>
-          <t>CLOISONNE ROUGE FLAMBE 440X</t>
+          <t>ENVASE VIDRIO ROSADO MARCADO 30ML</t>
         </is>
       </c>
       <c r="C1577" t="n">
-        <v>6266</v>
+        <v>46</v>
       </c>
       <c r="D1577" t="inlineStr"/>
       <c r="E1577" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1577" t="inlineStr">
@@ -40403,21 +40403,21 @@
     <row r="1589">
       <c r="A1589" t="inlineStr">
         <is>
-          <t>ET0202CA</t>
+          <t>190102</t>
         </is>
       </c>
       <c r="B1589" t="inlineStr">
         <is>
-          <t>ETIQUETA ILUMINADOR GOLD ROSE CARA</t>
+          <t>CARBÓN ACTIVADO</t>
         </is>
       </c>
       <c r="C1589" t="n">
-        <v>3916</v>
+        <v>500</v>
       </c>
       <c r="D1589" t="inlineStr"/>
       <c r="E1589" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F1589" t="inlineStr">
@@ -40429,21 +40429,21 @@
     <row r="1590">
       <c r="A1590" t="inlineStr">
         <is>
-          <t>190102</t>
+          <t>ET0202CA</t>
         </is>
       </c>
       <c r="B1590" t="inlineStr">
         <is>
-          <t>CARBÓN ACTIVADO</t>
+          <t>ETIQUETA ILUMINADOR GOLD ROSE CARA</t>
         </is>
       </c>
       <c r="C1590" t="n">
-        <v>500</v>
+        <v>3916</v>
       </c>
       <c r="D1590" t="inlineStr"/>
       <c r="E1590" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1590" t="inlineStr">
@@ -40507,21 +40507,21 @@
     <row r="1593">
       <c r="A1593" t="inlineStr">
         <is>
-          <t>ETC0160</t>
+          <t>ME0553</t>
         </is>
       </c>
       <c r="B1593" t="inlineStr">
         <is>
-          <t>CAJA RUBOR EN CREMA RUBY</t>
+          <t>TUBO COLAP TTO REVITALIZANTE 230ML V1</t>
         </is>
       </c>
       <c r="C1593" t="n">
-        <v>10536</v>
+        <v>478</v>
       </c>
       <c r="D1593" t="inlineStr"/>
       <c r="E1593" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1593" t="inlineStr">
@@ -40533,16 +40533,16 @@
     <row r="1594">
       <c r="A1594" t="inlineStr">
         <is>
-          <t>ETC0161</t>
+          <t>ETC0160</t>
         </is>
       </c>
       <c r="B1594" t="inlineStr">
         <is>
-          <t>CAJA RUBOR EN CREMA SALLY</t>
+          <t>CAJA RUBOR EN CREMA RUBY</t>
         </is>
       </c>
       <c r="C1594" t="n">
-        <v>10328</v>
+        <v>10536</v>
       </c>
       <c r="D1594" t="inlineStr"/>
       <c r="E1594" t="inlineStr">
@@ -40559,21 +40559,21 @@
     <row r="1595">
       <c r="A1595" t="inlineStr">
         <is>
-          <t>ME0553</t>
+          <t>ETC0161</t>
         </is>
       </c>
       <c r="B1595" t="inlineStr">
         <is>
-          <t>TUBO COLAP TTO REVITALIZANTE 230ML V1</t>
+          <t>CAJA RUBOR EN CREMA SALLY</t>
         </is>
       </c>
       <c r="C1595" t="n">
-        <v>478</v>
+        <v>10328</v>
       </c>
       <c r="D1595" t="inlineStr"/>
       <c r="E1595" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1595" t="inlineStr">
@@ -41105,21 +41105,21 @@
     <row r="1616">
       <c r="A1616" t="inlineStr">
         <is>
-          <t>ETC0173</t>
+          <t>ME0506</t>
         </is>
       </c>
       <c r="B1616" t="inlineStr">
         <is>
-          <t>CAJA TONICO CAPILAR KABA ROSADA 120ML</t>
+          <t>BALA TRANSPARENTE 260/250 ML</t>
         </is>
       </c>
       <c r="C1616" t="n">
-        <v>193</v>
+        <v>4464</v>
       </c>
       <c r="D1616" t="inlineStr"/>
       <c r="E1616" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1616" t="inlineStr">
@@ -41131,21 +41131,21 @@
     <row r="1617">
       <c r="A1617" t="inlineStr">
         <is>
-          <t>ME0506</t>
+          <t>ETC0173</t>
         </is>
       </c>
       <c r="B1617" t="inlineStr">
         <is>
-          <t>BALA TRANSPARENTE 260/250 ML</t>
+          <t>CAJA TONICO CAPILAR KABA ROSADA 120ML</t>
         </is>
       </c>
       <c r="C1617" t="n">
-        <v>4464</v>
+        <v>193</v>
       </c>
       <c r="D1617" t="inlineStr"/>
       <c r="E1617" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1617" t="inlineStr">
@@ -41261,16 +41261,16 @@
     <row r="1622">
       <c r="A1622" t="inlineStr">
         <is>
-          <t>ME1001VG</t>
+          <t>ME0515VG</t>
         </is>
       </c>
       <c r="B1622" t="inlineStr">
         <is>
-          <t>TAPA BRONCEADOR R/24 VIVIANA GRONDONA</t>
+          <t>ENVASE CAPSULA BRONCEADOR VIVIANA GRONDO</t>
         </is>
       </c>
       <c r="C1622" t="n">
-        <v>12219</v>
+        <v>11568</v>
       </c>
       <c r="D1622" t="inlineStr"/>
       <c r="E1622" t="inlineStr">
@@ -41287,16 +41287,16 @@
     <row r="1623">
       <c r="A1623" t="inlineStr">
         <is>
-          <t>ME0533VG</t>
+          <t>ME1001VG</t>
         </is>
       </c>
       <c r="B1623" t="inlineStr">
         <is>
-          <t>ENVASE Y TAPA APLICADOR VIVIANA GRONDONA</t>
+          <t>TAPA BRONCEADOR R/24 VIVIANA GRONDONA</t>
         </is>
       </c>
       <c r="C1623" t="n">
-        <v>11568</v>
+        <v>12219</v>
       </c>
       <c r="D1623" t="inlineStr"/>
       <c r="E1623" t="inlineStr">
@@ -41313,12 +41313,12 @@
     <row r="1624">
       <c r="A1624" t="inlineStr">
         <is>
-          <t>ME0515VG</t>
+          <t>ME0533VG</t>
         </is>
       </c>
       <c r="B1624" t="inlineStr">
         <is>
-          <t>ENVASE CAPSULA BRONCEADOR VIVIANA GRONDO</t>
+          <t>ENVASE Y TAPA APLICADOR VIVIANA GRONDONA</t>
         </is>
       </c>
       <c r="C1624" t="n">
@@ -45285,21 +45285,21 @@
     <row r="1773">
       <c r="A1773" t="inlineStr">
         <is>
-          <t>ET0204VG</t>
+          <t>144301</t>
         </is>
       </c>
       <c r="B1773" t="inlineStr">
         <is>
-          <t>ETIQUETA LIP GLOSS VIVIANA GRONDONA D2</t>
+          <t>ALCOHOL CETOESTEARÍLICO 30/70</t>
         </is>
       </c>
       <c r="C1773" t="n">
-        <v>2500</v>
+        <v>96090</v>
       </c>
       <c r="D1773" t="inlineStr"/>
       <c r="E1773" t="inlineStr">
         <is>
-          <t>MATERIAL DE ACONDICIONAMIENTO</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F1773" t="inlineStr">
@@ -45311,12 +45311,12 @@
     <row r="1774">
       <c r="A1774" t="inlineStr">
         <is>
-          <t>ET0203VG</t>
+          <t>ET0204VG</t>
         </is>
       </c>
       <c r="B1774" t="inlineStr">
         <is>
-          <t>ETIQUETA LIP GLOSS VIVIANA GRONDONA D1</t>
+          <t>ETIQUETA LIP GLOSS VIVIANA GRONDONA D2</t>
         </is>
       </c>
       <c r="C1774" t="n">
@@ -45337,21 +45337,21 @@
     <row r="1775">
       <c r="A1775" t="inlineStr">
         <is>
-          <t>144301</t>
+          <t>ET0203VG</t>
         </is>
       </c>
       <c r="B1775" t="inlineStr">
         <is>
-          <t>ALCOHOL CETOESTEARÍLICO 30/70</t>
+          <t>ETIQUETA LIP GLOSS VIVIANA GRONDONA D1</t>
         </is>
       </c>
       <c r="C1775" t="n">
-        <v>96090</v>
+        <v>2500</v>
       </c>
       <c r="D1775" t="inlineStr"/>
       <c r="E1775" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE ACONDICIONAMIENTO</t>
         </is>
       </c>
       <c r="F1775" t="inlineStr">
@@ -46767,16 +46767,16 @@
     <row r="1830">
       <c r="A1830" t="inlineStr">
         <is>
-          <t>ME0572</t>
+          <t>ME0544</t>
         </is>
       </c>
       <c r="B1830" t="inlineStr">
         <is>
-          <t>COLAPSIBLE AZUL CREMA CORPORAL ACLARANTE</t>
+          <t>TUBO COLAP DERMOACLARANTE 60ML V1</t>
         </is>
       </c>
       <c r="C1830" t="n">
-        <v>6750</v>
+        <v>815</v>
       </c>
       <c r="D1830" t="inlineStr"/>
       <c r="E1830" t="inlineStr">
@@ -46793,16 +46793,16 @@
     <row r="1831">
       <c r="A1831" t="inlineStr">
         <is>
-          <t>ME0544</t>
+          <t>ME0572</t>
         </is>
       </c>
       <c r="B1831" t="inlineStr">
         <is>
-          <t>TUBO COLAP DERMOACLARANTE 60ML V1</t>
+          <t>COLAPSIBLE AZUL CREMA CORPORAL ACLARANTE</t>
         </is>
       </c>
       <c r="C1831" t="n">
-        <v>815</v>
+        <v>6750</v>
       </c>
       <c r="D1831" t="inlineStr"/>
       <c r="E1831" t="inlineStr">

</xml_diff>

<commit_message>
Actualizar inventario_operaciones.xlsx (solo-inventario) - 2026-08-18 06:15
</commit_message>
<xml_diff>
--- a/inventario_operaciones.xlsx
+++ b/inventario_operaciones.xlsx
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>-128</v>
+        <v>140</v>
       </c>
       <c r="D18" t="n">
         <v>1701.068702290076</v>
@@ -7333,19 +7333,19 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>K010402</t>
+          <t>D030601</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>PERFUME PARA EL CABELLO CONFIDENTE KABA</t>
+          <t>FRESHING POP AFTER SUN DLUCHI</t>
         </is>
       </c>
       <c r="C253" t="n">
-        <v>2016</v>
+        <v>20136</v>
       </c>
       <c r="D253" t="n">
-        <v>1163.473282442748</v>
+        <v>267.9389312977099</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -7361,19 +7361,19 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>D030601</t>
+          <t>K010402</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>FRESHING POP AFTER SUN DLUCHI</t>
+          <t>PERFUME PARA EL CABELLO CONFIDENTE KABA</t>
         </is>
       </c>
       <c r="C254" t="n">
-        <v>20136</v>
+        <v>2016</v>
       </c>
       <c r="D254" t="n">
-        <v>267.9389312977099</v>
+        <v>1163.473282442748</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Actualizar inventario_operaciones.xlsx - 2026-09-07 05:58
</commit_message>
<xml_diff>
--- a/inventario_operaciones.xlsx
+++ b/inventario_operaciones.xlsx
@@ -9089,21 +9089,21 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>340302</t>
+          <t>ME0546</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>340302</t>
+          <t>TUBO COLAP FOTOPROTECTOR 60ML V1</t>
         </is>
       </c>
       <c r="C319" t="n">
-        <v>44000</v>
+        <v>4514</v>
       </c>
       <c r="D319" t="inlineStr"/>
       <c r="E319" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
@@ -9115,21 +9115,21 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>ME0546</t>
+          <t>340302</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>TUBO COLAP FOTOPROTECTOR 60ML V1</t>
+          <t>340302</t>
         </is>
       </c>
       <c r="C320" t="n">
-        <v>4514</v>
+        <v>44000</v>
       </c>
       <c r="D320" t="inlineStr"/>
       <c r="E320" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
@@ -36139,21 +36139,21 @@
     <row r="1425">
       <c r="A1425" t="inlineStr">
         <is>
-          <t>314208</t>
+          <t>ME1049</t>
         </is>
       </c>
       <c r="B1425" t="inlineStr">
         <is>
-          <t>GEMTONE AMBER G001</t>
+          <t>TAPA PUSH PULL DORADA ROSCA 24</t>
         </is>
       </c>
       <c r="C1425" t="n">
-        <v>73488</v>
+        <v>3386</v>
       </c>
       <c r="D1425" t="inlineStr"/>
       <c r="E1425" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1425" t="inlineStr">
@@ -36165,21 +36165,21 @@
     <row r="1426">
       <c r="A1426" t="inlineStr">
         <is>
-          <t>ME1049</t>
+          <t>314208</t>
         </is>
       </c>
       <c r="B1426" t="inlineStr">
         <is>
-          <t>TAPA PUSH PULL DORADA ROSCA 24</t>
+          <t>GEMTONE AMBER G001</t>
         </is>
       </c>
       <c r="C1426" t="n">
-        <v>3386</v>
+        <v>73488</v>
       </c>
       <c r="D1426" t="inlineStr"/>
       <c r="E1426" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F1426" t="inlineStr">
@@ -37517,21 +37517,21 @@
     <row r="1478">
       <c r="A1478" t="inlineStr">
         <is>
-          <t>173501</t>
+          <t>ME1043</t>
         </is>
       </c>
       <c r="B1478" t="inlineStr">
         <is>
-          <t>ULTRAMAR U-200 AZUL</t>
+          <t>TAPA FLIP TOP DORADA ROSCA 18</t>
         </is>
       </c>
       <c r="C1478" t="n">
-        <v>5025</v>
+        <v>2731</v>
       </c>
       <c r="D1478" t="inlineStr"/>
       <c r="E1478" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1478" t="inlineStr">
@@ -37543,16 +37543,16 @@
     <row r="1479">
       <c r="A1479" t="inlineStr">
         <is>
-          <t>ME1043</t>
+          <t>ME1044</t>
         </is>
       </c>
       <c r="B1479" t="inlineStr">
         <is>
-          <t>TAPA FLIP TOP DORADA ROSCA 18</t>
+          <t>TAPA FLIP TOP PLATEADA ROSCA 18</t>
         </is>
       </c>
       <c r="C1479" t="n">
-        <v>2731</v>
+        <v>39166</v>
       </c>
       <c r="D1479" t="inlineStr"/>
       <c r="E1479" t="inlineStr">
@@ -37569,21 +37569,21 @@
     <row r="1480">
       <c r="A1480" t="inlineStr">
         <is>
-          <t>ME1044</t>
+          <t>173501</t>
         </is>
       </c>
       <c r="B1480" t="inlineStr">
         <is>
-          <t>TAPA FLIP TOP PLATEADA ROSCA 18</t>
+          <t>ULTRAMAR U-200 AZUL</t>
         </is>
       </c>
       <c r="C1480" t="n">
-        <v>39166</v>
+        <v>5025</v>
       </c>
       <c r="D1480" t="inlineStr"/>
       <c r="E1480" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F1480" t="inlineStr">
@@ -38921,16 +38921,16 @@
     <row r="1532">
       <c r="A1532" t="inlineStr">
         <is>
-          <t>ME0507</t>
+          <t>ME0504</t>
         </is>
       </c>
       <c r="B1532" t="inlineStr">
         <is>
-          <t>BALA TRANSPARENTE 30ML</t>
+          <t>BALA NEGRA LARGA 120ML</t>
         </is>
       </c>
       <c r="C1532" t="n">
-        <v>24300</v>
+        <v>9239</v>
       </c>
       <c r="D1532" t="inlineStr"/>
       <c r="E1532" t="inlineStr">
@@ -38947,16 +38947,16 @@
     <row r="1533">
       <c r="A1533" t="inlineStr">
         <is>
-          <t>ME0504</t>
+          <t>ME1028</t>
         </is>
       </c>
       <c r="B1533" t="inlineStr">
         <is>
-          <t>BALA NEGRA LARGA 120ML</t>
+          <t>TAPA CON APLICADOR PUNTA PINCEL</t>
         </is>
       </c>
       <c r="C1533" t="n">
-        <v>9239</v>
+        <v>15877</v>
       </c>
       <c r="D1533" t="inlineStr"/>
       <c r="E1533" t="inlineStr">
@@ -38973,16 +38973,16 @@
     <row r="1534">
       <c r="A1534" t="inlineStr">
         <is>
-          <t>ME1028</t>
+          <t>ME1059</t>
         </is>
       </c>
       <c r="B1534" t="inlineStr">
         <is>
-          <t>TAPA CON APLICADOR PUNTA PINCEL</t>
+          <t>WIPER ( ESCURRIDOR/BARREDOR) NATURAL</t>
         </is>
       </c>
       <c r="C1534" t="n">
-        <v>15877</v>
+        <v>30387</v>
       </c>
       <c r="D1534" t="inlineStr"/>
       <c r="E1534" t="inlineStr">
@@ -38999,16 +38999,16 @@
     <row r="1535">
       <c r="A1535" t="inlineStr">
         <is>
-          <t>ME1059</t>
+          <t>ME0507</t>
         </is>
       </c>
       <c r="B1535" t="inlineStr">
         <is>
-          <t>WIPER ( ESCURRIDOR/BARREDOR) NATURAL</t>
+          <t>BALA TRANSPARENTE 30ML</t>
         </is>
       </c>
       <c r="C1535" t="n">
-        <v>30387</v>
+        <v>24300</v>
       </c>
       <c r="D1535" t="inlineStr"/>
       <c r="E1535" t="inlineStr">
@@ -41543,21 +41543,21 @@
     <row r="1633">
       <c r="A1633" t="inlineStr">
         <is>
-          <t>314202</t>
+          <t>ME0527</t>
         </is>
       </c>
       <c r="B1633" t="inlineStr">
         <is>
-          <t>CLOISONNE ROUGE FLAMBE 440X</t>
+          <t>ENVASE VIDRIO ROSADO MARCADO 30ML</t>
         </is>
       </c>
       <c r="C1633" t="n">
-        <v>6266</v>
+        <v>46</v>
       </c>
       <c r="D1633" t="inlineStr"/>
       <c r="E1633" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F1633" t="inlineStr">
@@ -41569,21 +41569,21 @@
     <row r="1634">
       <c r="A1634" t="inlineStr">
         <is>
-          <t>ME0527</t>
+          <t>314202</t>
         </is>
       </c>
       <c r="B1634" t="inlineStr">
         <is>
-          <t>ENVASE VIDRIO ROSADO MARCADO 30ML</t>
+          <t>CLOISONNE ROUGE FLAMBE 440X</t>
         </is>
       </c>
       <c r="C1634" t="n">
-        <v>46</v>
+        <v>6266</v>
       </c>
       <c r="D1634" t="inlineStr"/>
       <c r="E1634" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F1634" t="inlineStr">
@@ -51551,21 +51551,21 @@
     <row r="2011">
       <c r="A2011" t="inlineStr">
         <is>
-          <t>173501</t>
+          <t>ME1043</t>
         </is>
       </c>
       <c r="B2011" t="inlineStr">
         <is>
-          <t>ULTRAMAR U-200 AZUL</t>
+          <t>TAPA FLIP TOP DORADA ROSCA 18</t>
         </is>
       </c>
       <c r="C2011" t="n">
-        <v>309</v>
+        <v>3588</v>
       </c>
       <c r="D2011" t="inlineStr"/>
       <c r="E2011" t="inlineStr">
         <is>
-          <t>MATERIA PRIMA</t>
+          <t>MATERIAL DE EMPAQUE</t>
         </is>
       </c>
       <c r="F2011" t="inlineStr">
@@ -51577,21 +51577,21 @@
     <row r="2012">
       <c r="A2012" t="inlineStr">
         <is>
-          <t>ME1043</t>
+          <t>173501</t>
         </is>
       </c>
       <c r="B2012" t="inlineStr">
         <is>
-          <t>TAPA FLIP TOP DORADA ROSCA 18</t>
+          <t>ULTRAMAR U-200 AZUL</t>
         </is>
       </c>
       <c r="C2012" t="n">
-        <v>3588</v>
+        <v>309</v>
       </c>
       <c r="D2012" t="inlineStr"/>
       <c r="E2012" t="inlineStr">
         <is>
-          <t>MATERIAL DE EMPAQUE</t>
+          <t>MATERIA PRIMA</t>
         </is>
       </c>
       <c r="F2012" t="inlineStr">

</xml_diff>